<commit_message>
Trim the work from the Welcome and Early Access openers
The Welcome email now says "Our upcoming collaboration with {artist} is the
latest in this lineage." and runs straight into the guides line; the timed
Early Access opener stops at "for {window} only." The hook that follows names
the work, so the "– title, edition phrase" tail is gone from both, and the
optional short hook with it. Same change in the workbook and the template.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KCpXfXvgVaMZkSdhMYLgwy
</commit_message>
<xml_diff>
--- a/tool/release-copy.xlsx
+++ b/tool/release-copy.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="B39" s="10">
-        <f>IF(OR($B$16="",$B$43),"",", released in support of "&amp;$B$16)</f>
+        <f>IF(OR($B$16="",$B$42),"",", released in support of "&amp;$B$16)</f>
         <v/>
       </c>
     </row>
@@ -1050,231 +1050,253 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>hook_short</t>
+          <t>hook_names_beneficiary</t>
         </is>
       </c>
       <c r="B42" s="10">
-        <f>IF(ISNUMBER(FIND(". ",$B$28)),LEFT($B$28,FIND(". ",$B$28)),$B$28)</f>
+        <f>IF($B$16="",FALSE,ISNUMBER(SEARCH($B$16,$B$28)))</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>hook_names_beneficiary</t>
+          <t>features</t>
         </is>
       </c>
       <c r="B43" s="10">
-        <f>IF($B$16="",FALSE,ISNUMBER(SEARCH($B$16,$B$28)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
+        <f>$B$20&amp;IF($B$21="","",". "&amp;$B$21)&amp;IF($B$22="","",". "&amp;$B$22)&amp;IF($B$23="","",". "&amp;$B$23)&amp;IF($B$24="","",". "&amp;$B$24)&amp;"."</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="60" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>features</t>
+          <t>features_list</t>
         </is>
       </c>
       <c r="B44" s="10">
-        <f>$B$20&amp;IF($B$21="","",". "&amp;$B$21)&amp;IF($B$22="","",". "&amp;$B$22)&amp;IF($B$23="","",". "&amp;$B$23)&amp;IF($B$24="","",". "&amp;$B$24)&amp;"."</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" ht="60" customHeight="1">
+        <f>"· "&amp;$B$20&amp;IF($B$21="","",CHAR(10)&amp;"· "&amp;$B$21)&amp;IF($B$22="","",CHAR(10)&amp;"· "&amp;$B$22)&amp;IF($B$23="","",CHAR(10)&amp;"· "&amp;$B$23)&amp;IF($B$24="","",CHAR(10)&amp;"· "&amp;$B$24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" ht="70" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>features_list</t>
+          <t>features_list_support</t>
         </is>
       </c>
       <c r="B45" s="10">
-        <f>"· "&amp;$B$20&amp;IF($B$21="","",CHAR(10)&amp;"· "&amp;$B$21)&amp;IF($B$22="","",CHAR(10)&amp;"· "&amp;$B$22)&amp;IF($B$23="","",CHAR(10)&amp;"· "&amp;$B$23)&amp;IF($B$24="","",CHAR(10)&amp;"· "&amp;$B$24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" ht="70" customHeight="1">
+        <f>$B$44&amp;IF(OR($B$16="",$B$42),"",CHAR(10)&amp;"· Released in support of "&amp;$B$16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>features_list_support</t>
+          <t>making_ours</t>
         </is>
       </c>
       <c r="B46" s="10">
-        <f>$B$45&amp;IF(OR($B$16="",$B$43),"",CHAR(10)&amp;"· Released in support of "&amp;$B$16)</f>
+        <f>SUBSTITUTE($B$29,"printmakers at Make-Ready","our printmakers at Make-Ready")</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>making_ours</t>
+          <t>making_ours_tagged</t>
         </is>
       </c>
       <c r="B47" s="10">
-        <f>SUBSTITUTE($B$29,"printmakers at Make-Ready","our printmakers at Make-Ready")</f>
+        <f>SUBSTITUTE($B$29,"printmakers at Make-Ready","our printmakers at Make-Ready (@make__ready)")</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>making_ours_tagged</t>
+          <t>launch_date</t>
         </is>
       </c>
       <c r="B48" s="10">
-        <f>SUBSTITUTE($B$29,"printmakers at Make-Ready","our printmakers at Make-Ready (@make__ready)")</f>
+        <f>TEXT($B$14,"d mmmm")</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>launch_date</t>
+          <t>launch_time</t>
         </is>
       </c>
       <c r="B49" s="10">
-        <f>TEXT($B$14,"d mmmm")</f>
+        <f>TEXT($B$14,"hh:mm")&amp;" UK time"</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>launch_time</t>
+          <t>launch_weekday</t>
         </is>
       </c>
       <c r="B50" s="10">
-        <f>TEXT($B$14,"hh:mm")&amp;" UK time"</f>
+        <f>TEXT($B$14,"dddd")</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>launch_weekday</t>
+          <t>launch_date_dd</t>
         </is>
       </c>
       <c r="B51" s="10">
-        <f>TEXT($B$14,"dddd")</f>
+        <f>TEXT($B$14,"dd mmmm")</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>launch_date_dd</t>
+          <t>close_date</t>
         </is>
       </c>
       <c r="B52" s="10">
-        <f>TEXT($B$14,"dd mmmm")</f>
+        <f>TEXT($B$15,"d mmmm")</f>
         <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>close_date</t>
+          <t>close_time</t>
         </is>
       </c>
       <c r="B53" s="10">
-        <f>TEXT($B$15,"d mmmm")</f>
+        <f>TEXT($B$15,"hh:mm")&amp;" UK time"</f>
         <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>close_time</t>
+          <t>close_weekday</t>
         </is>
       </c>
       <c r="B54" s="10">
-        <f>TEXT($B$15,"hh:mm")&amp;" UK time"</f>
+        <f>TEXT($B$15,"dddd")</f>
         <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>close_weekday</t>
+          <t>close_date_dd</t>
         </is>
       </c>
       <c r="B55" s="10">
-        <f>TEXT($B$15,"dddd")</f>
+        <f>TEXT($B$15,"dd mmmm")</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>close_date_dd</t>
+          <t>collect_phrase</t>
         </is>
       </c>
       <c r="B56" s="10">
-        <f>TEXT($B$15,"dd mmmm")</f>
+        <f>SUBSTITUTE($B$10," new "," ")</f>
         <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>collect_phrase</t>
+          <t>edition_phrase_cap</t>
         </is>
       </c>
       <c r="B57" s="10">
-        <f>SUBSTITUTE($B$10," new "," ")</f>
+        <f>UPPER(LEFT($B$10,1))&amp;MID($B$10,2,999)</f>
         <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>edition_phrase_cap</t>
+          <t>window_cap</t>
         </is>
       </c>
       <c r="B58" s="10">
-        <f>UPPER(LEFT($B$10,1))&amp;MID($B$10,2,999)</f>
+        <f>UPPER(LEFT($B$13,1))&amp;MID($B$13,2,999)</f>
         <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>window_cap</t>
+          <t>card_line</t>
         </is>
       </c>
       <c r="B59" s="10">
-        <f>UPPER(LEFT($B$13,1))&amp;MID($B$13,2,999)</f>
+        <f>$B$57&amp;" by "&amp;$B$4&amp;"."</f>
         <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>card_line</t>
+          <t>card</t>
         </is>
       </c>
       <c r="B60" s="10">
-        <f>$B$58&amp;" by "&amp;$B$4&amp;"."</f>
+        <f>$B$8&amp;CHAR(10)&amp;$B$59</f>
         <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>quote_line</t>
         </is>
       </c>
       <c r="B61" s="10">
-        <f>$B$8&amp;CHAR(10)&amp;$B$60</f>
+        <f>IF($B$30="","","“"&amp;$B$30&amp;"” – "&amp;$B$4)</f>
         <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>quote_line</t>
+          <t>each_artwork</t>
         </is>
       </c>
       <c r="B62" s="10">
-        <f>IF($B$30="","","“"&amp;$B$30&amp;"” – "&amp;$B$4)</f>
+        <f>IF($B$11&gt;1," for each artwork","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>work_word</t>
+        </is>
+      </c>
+      <c r="B63" s="10">
+        <f>IF($B$11&gt;1,"works","work")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>add_what</t>
+        </is>
+      </c>
+      <c r="B64" s="10">
+        <f>IF($B$11&gt;1,"a print",$B$36)</f>
         <v/>
       </c>
     </row>
@@ -1289,7 +1311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1507,7 +1529,7 @@
         </is>
       </c>
       <c r="C15" s="10">
-        <f>SUBSTITUTE(B15,"{features}",Inputs!$B$44)</f>
+        <f>SUBSTITUTE(B15,"{features}",Inputs!$B$43)</f>
         <v/>
       </c>
     </row>
@@ -1539,7 +1561,7 @@
         </is>
       </c>
       <c r="C17" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17,"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$49),"{launch_time}",Inputs!$B$50)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17,"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$48),"{launch_time}",Inputs!$B$49)</f>
         <v/>
       </c>
     </row>
@@ -1555,7 +1577,7 @@
         </is>
       </c>
       <c r="C18" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B18,"{close_date}",Inputs!$B$53),"{close_time}",Inputs!$B$54)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B18,"{close_date}",Inputs!$B$52),"{close_time}",Inputs!$B$53)</f>
         <v/>
       </c>
     </row>
@@ -1571,7 +1593,7 @@
         </is>
       </c>
       <c r="C19" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B19,"{close_date}",Inputs!$B$53),"{close_time}",Inputs!$B$54)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B19,"{close_date}",Inputs!$B$52),"{close_time}",Inputs!$B$53)</f>
         <v/>
       </c>
     </row>
@@ -1587,7 +1609,7 @@
         </is>
       </c>
       <c r="C20" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B20,"{close_date}",Inputs!$B$53),"{close_time}",Inputs!$B$54)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B20,"{close_date}",Inputs!$B$52),"{close_time}",Inputs!$B$53)</f>
         <v/>
       </c>
     </row>
@@ -1674,7 +1696,7 @@
         </is>
       </c>
       <c r="C26" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B26,"{close_date}",Inputs!$B$53),"{close_time}",Inputs!$B$54)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B26,"{close_date}",Inputs!$B$52),"{close_time}",Inputs!$B$53)</f>
         <v/>
       </c>
     </row>
@@ -1713,7 +1735,7 @@
         </is>
       </c>
       <c r="C29" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B29,"{artist}",Inputs!$B$4),"{edition_phrase_cap}",Inputs!$B$58)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B29,"{artist}",Inputs!$B$4),"{edition_phrase_cap}",Inputs!$B$57)</f>
         <v/>
       </c>
     </row>
@@ -1745,7 +1767,7 @@
         </is>
       </c>
       <c r="C31" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B31,"{window}",Inputs!$B$13),"{launch_time}",Inputs!$B$50),"{launch_weekday}",Inputs!$B$51),"{launch_date_dd}",Inputs!$B$52)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B31,"{window}",Inputs!$B$13),"{launch_time}",Inputs!$B$49),"{launch_weekday}",Inputs!$B$50),"{launch_date_dd}",Inputs!$B$51)</f>
         <v/>
       </c>
     </row>
@@ -1804,7 +1826,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="32" customHeight="1">
+    <row r="36" ht="64" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
           <t>email · welcome · 3</t>
@@ -1812,15 +1834,15 @@
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>Our upcoming collaboration with {artist} is the latest in this lineage – {work_intro}. {hook_short}</t>
+          <t>Our upcoming collaboration with {artist} is the latest in this lineage. If you're new to collecting art or curious about limited editions, our library of guides is a good place to start. In particular, How to collect art and What is an edition?</t>
         </is>
       </c>
       <c r="C36" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B36,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$38),"{hook_short}",Inputs!$B$42)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="48" customHeight="1">
+        <f>SUBSTITUTE(B36,"{artist}",Inputs!$B$4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="32" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
           <t>email · welcome · 4</t>
@@ -1828,7 +1850,7 @@
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>If you're new to collecting art or curious about limited editions, our library of guides is a good place to start. In particular, How to collect art and What is an edition?</t>
+          <t>Let us know if you have any questions. We're excited to see what you collect.</t>
         </is>
       </c>
       <c r="C37" s="10">
@@ -1836,54 +1858,54 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="32" customHeight="1">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>email · welcome · 5</t>
-        </is>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>Let us know if you have any questions. We're excited to see what you collect.</t>
-        </is>
-      </c>
-      <c r="C38" s="10">
-        <f>B38</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>EMAILS · early access</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="48" customHeight="1">
+    <row r="39" ht="32" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>email · early access, timed · opener</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>Our {ordinal} collaboration with {artist} launches tomorrow at {launch_time} and will be available to collect for {window} only.</t>
+        </is>
+      </c>
+      <c r="C39" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B39,"{artist}",Inputs!$B$4),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_time}",Inputs!$B$49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="32" customHeight="1">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>email · early access, timed · opener</t>
+          <t>email · early access, timed · registered line</t>
         </is>
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>Our {ordinal} collaboration with {artist} launches tomorrow at {launch_time} and will be available to collect for {window} only – {work_intro}.</t>
+          <t>As a thank you for registering for updates, we're offering you the chance to collect the release 24 hours before everyone else.</t>
         </is>
       </c>
       <c r="C40" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B40,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$38),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_time}",Inputs!$B$50)</f>
+        <f>B40</f>
         <v/>
       </c>
     </row>
     <row r="41" ht="32" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>email · early access, timed · registered line</t>
+          <t>email · early access, timed · past collectors line</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>As a thank you for registering for updates, we're offering you the chance to collect the release 24 hours before everyone else.</t>
+          <t>As a previous collector of the artist, we're offering you the chance to order the collaboration 24 hours before everyone else.</t>
         </is>
       </c>
       <c r="C41" s="10">
@@ -1891,15 +1913,15 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="32" customHeight="1">
+    <row r="42" ht="16" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>email · early access, timed · past collectors line</t>
+          <t>email · early access, timed · unlock line</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>As a previous collector of the artist, we're offering you the chance to order the collaboration 24 hours before everyone else.</t>
+          <t>Unlock early access using the link below.</t>
         </is>
       </c>
       <c r="C42" s="10">
@@ -1907,232 +1929,232 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="16" customHeight="1">
+    <row r="43" ht="32" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>email · early access, timed · unlock line</t>
+          <t>email · early access, draw · 1</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>Unlock early access using the link below.</t>
+          <t>We're currently preparing the launch of our {ordinal} collaboration with {artist} – {work_intro}{support}.</t>
         </is>
       </c>
       <c r="C43" s="10">
-        <f>B43</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" ht="32" customHeight="1">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B43,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$38),"{support}",Inputs!$B$39),"{ordinal}",Inputs!$B$7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="96" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>email · early access, draw · 1</t>
+          <t>email · early access, draw · 2</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>We're currently preparing the launch of our {ordinal} collaboration with {artist} – {work_intro}{support}.</t>
+          <t>The edition will launch publicly on {launch_date} and will be allocated by a randomised draw; however, for the next 48 hours we're offering a small group of collectors a first look, plus access to a limited number of pre-orders. Based on your order history and the artists you've expressed an interest in, I thought the edition would be a good fit for your collection.</t>
         </is>
       </c>
       <c r="C44" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B44,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$38),"{support}",Inputs!$B$39),"{ordinal}",Inputs!$B$7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" ht="96" customHeight="1">
+        <f>SUBSTITUTE(B44,"{launch_date}",Inputs!$B$48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" ht="32" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>email · early access, draw · 2</t>
+          <t>email · early access, draw · 3</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>The edition will launch publicly on {launch_date} and will be allocated by a randomised draw; however, for the next 48 hours we're offering a small group of collectors a first look, plus access to a limited number of pre-orders. Based on your order history and the artists you've expressed an interest in, I thought the edition would be a good fit for your collection.</t>
+          <t>Explore the artwork and place your order via the private link below. Use code {early_access_code} to unlock early access.</t>
         </is>
       </c>
       <c r="C45" s="10">
-        <f>SUBSTITUTE(B45,"{launch_date}",Inputs!$B$49)</f>
+        <f>SUBSTITUTE(B45,"{early_access_code}",Inputs!$B$19)</f>
         <v/>
       </c>
     </row>
     <row r="46" ht="32" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>email · early access, draw · 3</t>
+          <t>email · insiders · opener</t>
         </is>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Explore the artwork and place your order via the private link below. Use code {early_access_code} to unlock early access.</t>
+          <t>I'm delighted to share our {ordinal} collaboration with {artist} – {work_intro}{support}.</t>
         </is>
       </c>
       <c r="C46" s="10">
-        <f>SUBSTITUTE(B46,"{early_access_code}",Inputs!$B$19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" ht="32" customHeight="1">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B46,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$38),"{support}",Inputs!$B$39),"{ordinal}",Inputs!$B$7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="64" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>email · insiders · opener</t>
+          <t>email · insiders · mechanics, draw</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
         <is>
-          <t>I'm delighted to share our {ordinal} collaboration with {artist} – {work_intro}{support}.</t>
+          <t>The edition will launch publicly on {launch_date} and will be allocated by a randomised draw. However, for the next 48 hours, I'm excited to offer you a first look, plus early access to a limited number of pre-orders.</t>
         </is>
       </c>
       <c r="C47" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B47,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$38),"{support}",Inputs!$B$39),"{ordinal}",Inputs!$B$7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" ht="64" customHeight="1">
+        <f>SUBSTITUTE(B47,"{launch_date}",Inputs!$B$48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="48" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>email · insiders · mechanics, draw</t>
+          <t>email · insiders · mechanics, timed</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>The edition will launch publicly on {launch_date} and will be allocated by a randomised draw. However, for the next 48 hours, I'm excited to offer you a first look, plus early access to a limited number of pre-orders.</t>
+          <t>The edition launches tomorrow at {launch_time} and will be available to collect for {window} only. For the next 24 hours, I'm excited to offer you early access ahead of the public launch.</t>
         </is>
       </c>
       <c r="C48" s="10">
-        <f>SUBSTITUTE(B48,"{launch_date}",Inputs!$B$49)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" ht="48" customHeight="1">
+        <f>SUBSTITUTE(SUBSTITUTE(B48,"{window}",Inputs!$B$13),"{launch_time}",Inputs!$B$49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="32" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>email · insiders · mechanics, timed</t>
+          <t>email · insiders · code line, draw</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>The edition launches tomorrow at {launch_time} and will be available to collect for {window} only. For the next 24 hours, I'm excited to offer you early access ahead of the public launch.</t>
+          <t>Discover the artwork and place your order via the private link below. Use code {early_access_code} to unlock early access.</t>
         </is>
       </c>
       <c r="C49" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B49,"{window}",Inputs!$B$13),"{launch_time}",Inputs!$B$50)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" ht="32" customHeight="1">
+        <f>SUBSTITUTE(B49,"{early_access_code}",Inputs!$B$19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="16" customHeight="1">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>email · insiders · code line, draw</t>
+          <t>email · insiders · link line, timed</t>
         </is>
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>Discover the artwork and place your order via the private link below. Use code {early_access_code} to unlock early access.</t>
+          <t>Discover the artwork and place your order via the private link below.</t>
         </is>
       </c>
       <c r="C50" s="10">
-        <f>SUBSTITUTE(B50,"{early_access_code}",Inputs!$B$19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" ht="16" customHeight="1">
+        <f>B50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="64" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>email · insiders · link line, timed</t>
+          <t>email · insiders · sign-off</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
-        <is>
-          <t>Discover the artwork and place your order via the private link below.</t>
-        </is>
-      </c>
-      <c r="C51" s="10">
-        <f>B51</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" ht="64" customHeight="1">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>email · insiders · sign-off</t>
-        </is>
-      </c>
-      <c r="B52" s="8" t="inlineStr">
         <is>
           <t>Best regards,
 {advisor}
 Art Advisor at Avant Arte</t>
         </is>
       </c>
-      <c r="C52" s="10">
-        <f>SUBSTITUTE(B52,"{advisor}",Inputs!$B$18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
+      <c r="C51" s="10">
+        <f>SUBSTITUTE(B51,"{advisor}",Inputs!$B$18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
         <is>
           <t>EMAILS · the window (TL)</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="32" customHeight="1">
+    <row r="53" ht="32" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>email · live · opener</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>Our {ordinal} collaboration with {artist} is now available to collect for {window} only – {work_intro}{support}.</t>
+        </is>
+      </c>
+      <c r="C53" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B53,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$38),"{support}",Inputs!$B$39),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" ht="48" customHeight="1">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>email · live · opener</t>
+          <t>email · live · closing line</t>
         </is>
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>Our {ordinal} collaboration with {artist} is now available to collect for {window} only – {work_intro}{support}.</t>
+          <t>The opportunity to collect an edition ends at {close_time} on {close_weekday}, {close_date_dd}. Click the link below to add {add_what} to your collection.</t>
         </is>
       </c>
       <c r="C54" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B54,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$38),"{support}",Inputs!$B$39),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55" ht="48" customHeight="1">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B54,"{close_time}",Inputs!$B$53),"{close_weekday}",Inputs!$B$54),"{close_date_dd}",Inputs!$B$55),"{add_what}",Inputs!$B$64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="16" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>email · live · closing line</t>
+          <t>email · halfway · kicker</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>The opportunity to collect an edition ends at {close_time} on {close_weekday}, {close_date_dd}. Click the link below to add {work_email} to your collection.</t>
+          <t>Collect a print by {artist}</t>
         </is>
       </c>
       <c r="C55" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B55,"{work_email}",Inputs!$B$36),"{close_time}",Inputs!$B$54),"{close_weekday}",Inputs!$B$55),"{close_date_dd}",Inputs!$B$56)</f>
+        <f>SUBSTITUTE(B55,"{artist}",Inputs!$B$4)</f>
         <v/>
       </c>
     </row>
     <row r="56" ht="16" customHeight="1">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>email · halfway · kicker</t>
+          <t>email · halfway · headline</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>Collect a print by {artist}</t>
+          <t>24 hours down, 24 to go</t>
         </is>
       </c>
       <c r="C56" s="10">
-        <f>SUBSTITUTE(B56,"{artist}",Inputs!$B$4)</f>
+        <f>B56</f>
         <v/>
       </c>
     </row>
     <row r="57" ht="16" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>email · halfway · headline</t>
+          <t>email · halfway · footer</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>24 hours down, 24 to go</t>
+          <t>There's still time to add a print to your collection.</t>
         </is>
       </c>
       <c r="C57" s="10">
@@ -2143,12 +2165,12 @@
     <row r="58" ht="16" customHeight="1">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>email · halfway · footer</t>
+          <t>email · 5 days · headline</t>
         </is>
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>There's still time to add a print to your collection.</t>
+          <t>2 days down, 5 days to go</t>
         </is>
       </c>
       <c r="C58" s="10">
@@ -2159,12 +2181,12 @@
     <row r="59" ht="16" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>email · 5 days · headline</t>
+          <t>email · 5 days · footer</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>2 days down, 5 days to go</t>
+          <t>Add a signed print to your collection</t>
         </is>
       </c>
       <c r="C59" s="10">
@@ -2175,12 +2197,12 @@
     <row r="60" ht="16" customHeight="1">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>email · 5 days · footer</t>
+          <t>email · 3 days · headline</t>
         </is>
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>Add a signed print to your collection</t>
+          <t>Three days left to collect</t>
         </is>
       </c>
       <c r="C60" s="10">
@@ -2188,205 +2210,205 @@
         <v/>
       </c>
     </row>
-    <row r="61" ht="16" customHeight="1">
+    <row r="61" ht="32" customHeight="1">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>email · 3 days · headline</t>
+          <t>email · 3 days · 1</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>Three days left to collect</t>
+          <t>There are just three days left to collect {collect_phrase} by {artist}.</t>
         </is>
       </c>
       <c r="C61" s="10">
-        <f>B61</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B61,"{artist}",Inputs!$B$4),"{collect_phrase}",Inputs!$B$56)</f>
         <v/>
       </c>
     </row>
     <row r="62" ht="32" customHeight="1">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>email · 3 days · 1</t>
+          <t>email · 3 days · 2</t>
         </is>
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>There are just three days left to collect {collect_phrase} by {artist}.</t>
+          <t>Click the link to collect before {close_time} on {close_weekday}, {close_date_dd}.</t>
         </is>
       </c>
       <c r="C62" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B62,"{artist}",Inputs!$B$4),"{collect_phrase}",Inputs!$B$57)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" ht="32" customHeight="1">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B62,"{close_time}",Inputs!$B$53),"{close_weekday}",Inputs!$B$54),"{close_date_dd}",Inputs!$B$55)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" ht="16" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>email · 3 days · 2</t>
+          <t>email · 3 days · footer</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>Click the link to collect before {close_time} on {close_weekday}, {close_date_dd}.</t>
+          <t>Add a print to your collection</t>
         </is>
       </c>
       <c r="C63" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B63,"{close_time}",Inputs!$B$54),"{close_weekday}",Inputs!$B$55),"{close_date_dd}",Inputs!$B$56)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64" ht="16" customHeight="1">
-      <c r="A64" s="4" t="inlineStr">
-        <is>
-          <t>email · 3 days · footer</t>
-        </is>
-      </c>
-      <c r="B64" s="8" t="inlineStr">
-        <is>
-          <t>Add a print to your collection</t>
-        </is>
-      </c>
-      <c r="C64" s="10">
-        <f>B64</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="3" t="inlineStr">
+        <f>B63</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
         <is>
           <t>EMAILS · last chance</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="48" customHeight="1">
+    <row r="65" ht="48" customHeight="1">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>email · last chance, timed · 1</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>It's now or never for our {ordinal} collaboration with {artist} – {collect_phrase} will be available to order until {close_time} on {close_weekday}, {close_date_dd}.</t>
+        </is>
+      </c>
+      <c r="C65" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B65,"{artist}",Inputs!$B$4),"{collect_phrase}",Inputs!$B$56),"{ordinal}",Inputs!$B$7),"{close_time}",Inputs!$B$53),"{close_weekday}",Inputs!$B$54),"{close_date_dd}",Inputs!$B$55)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" ht="32" customHeight="1">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>email · last chance, timed · 1</t>
+          <t>email · last chance, timed · 2</t>
         </is>
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>It's now or never for our {ordinal} collaboration with {artist} – {collect_phrase} will be available to order until {close_time} on {close_weekday}, {close_date_dd}.</t>
+          <t>After this time, the edition size{each_artwork} will be confirmed, and the {work_word} will no longer be available to purchase.</t>
         </is>
       </c>
       <c r="C66" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B66,"{artist}",Inputs!$B$4),"{collect_phrase}",Inputs!$B$57),"{ordinal}",Inputs!$B$7),"{close_time}",Inputs!$B$54),"{close_weekday}",Inputs!$B$55),"{close_date_dd}",Inputs!$B$56)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B66,"{each_artwork}",Inputs!$B$62),"{work_word}",Inputs!$B$63)</f>
         <v/>
       </c>
     </row>
     <row r="67" ht="32" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>email · last chance, timed · 2</t>
+          <t>email · last chance, draw · 1</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>After this time, the edition size will be confirmed, and the work will no longer be available to purchase.</t>
+          <t>This is your final opportunity to enter the draw for {work_email}, {collect_phrase} by {artist}.</t>
         </is>
       </c>
       <c r="C67" s="10">
-        <f>B67</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B67,"{artist}",Inputs!$B$4),"{work_email}",Inputs!$B$36),"{collect_phrase}",Inputs!$B$56)</f>
         <v/>
       </c>
     </row>
     <row r="68" ht="32" customHeight="1">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>email · last chance, draw · 1</t>
+          <t>email · last chance, draw · 2</t>
         </is>
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>This is your final opportunity to enter the draw for {work_email}, {collect_phrase} by {artist}.</t>
+          <t>For a chance to collect, click the link below to enter the draw. The draw closes at {close_time} on {close_weekday}, {close_date_dd}.</t>
         </is>
       </c>
       <c r="C68" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B68,"{artist}",Inputs!$B$4),"{work_email}",Inputs!$B$36),"{collect_phrase}",Inputs!$B$57)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69" ht="32" customHeight="1">
-      <c r="A69" s="4" t="inlineStr">
-        <is>
-          <t>email · last chance, draw · 2</t>
-        </is>
-      </c>
-      <c r="B69" s="8" t="inlineStr">
-        <is>
-          <t>For a chance to collect, click the link below to enter the draw. The draw closes at {close_time} on {close_weekday}, {close_date_dd}.</t>
-        </is>
-      </c>
-      <c r="C69" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B69,"{close_time}",Inputs!$B$54),"{close_weekday}",Inputs!$B$55),"{close_date_dd}",Inputs!$B$56)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="3" t="inlineStr">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B68,"{close_time}",Inputs!$B$53),"{close_weekday}",Inputs!$B$54),"{close_date_dd}",Inputs!$B$55)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
         <is>
           <t>EMAILS · surveys (LE)</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="16" customHeight="1">
+    <row r="70" ht="16" customHeight="1">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>email · first-time survey · subject</t>
+        </is>
+      </c>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>Congratulations on your first Avant Arte edition</t>
+        </is>
+      </c>
+      <c r="C70" s="10">
+        <f>B70</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="32" customHeight="1">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>email · first-time survey · subject</t>
+          <t>email · first-time survey · 1</t>
         </is>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>Congratulations on your first Avant Arte edition</t>
+          <t>Thank you for adding our collaboration with {artist} to your collection. Great choice!</t>
         </is>
       </c>
       <c r="C71" s="10">
-        <f>B71</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72" ht="32" customHeight="1">
+        <f>SUBSTITUTE(B71,"{artist}",Inputs!$B$4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72" ht="48" customHeight="1">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>email · first-time survey · 1</t>
+          <t>email · first-time survey · 2</t>
         </is>
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>Thank you for adding our collaboration with {artist} to your collection. Great choice!</t>
+          <t>I'm {advisor}, an art advisor at Avant Arte. I'm here to connect collectors with artists by making suggestions, answering questions and offering early access to our collaborations.</t>
         </is>
       </c>
       <c r="C72" s="10">
-        <f>SUBSTITUTE(B72,"{artist}",Inputs!$B$4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73" ht="48" customHeight="1">
+        <f>SUBSTITUTE(B72,"{advisor}",Inputs!$B$18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="32" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>email · first-time survey · 2</t>
+          <t>email · first-time survey · 3</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>I'm {advisor}, an art advisor at Avant Arte. I'm here to connect collectors with artists by making suggestions, answering questions and offering early access to our collaborations.</t>
+          <t>If you have two minutes to complete a short survey about your collecting journey to date, your responses will help guide my recommendations.</t>
         </is>
       </c>
       <c r="C73" s="10">
-        <f>SUBSTITUTE(B73,"{advisor}",Inputs!$B$18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74" ht="32" customHeight="1">
+        <f>B73</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="16" customHeight="1">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>email · first-time survey · 3</t>
+          <t>email · first-time survey · 4</t>
         </is>
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>If you have two minutes to complete a short survey about your collecting journey to date, your responses will help guide my recommendations.</t>
+          <t>Any questions? Reply to this email.</t>
         </is>
       </c>
       <c r="C74" s="10">
@@ -2394,47 +2416,47 @@
         <v/>
       </c>
     </row>
-    <row r="75" ht="16" customHeight="1">
+    <row r="75" ht="48" customHeight="1">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>email · first-time survey · 4</t>
+          <t>email · non-purchaser survey · 1</t>
         </is>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>Any questions? Reply to this email.</t>
+          <t>As someone who registered for updates but ultimately decided not to enter the draw for our collaboration with {artist}, we'd love your feedback.</t>
         </is>
       </c>
       <c r="C75" s="10">
-        <f>B75</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76" ht="48" customHeight="1">
+        <f>SUBSTITUTE(B75,"{artist}",Inputs!$B$4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76" ht="32" customHeight="1">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>email · non-purchaser survey · 1</t>
+          <t>email · non-purchaser survey · 2</t>
         </is>
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>As someone who registered for updates but ultimately decided not to enter the draw for our collaboration with {artist}, we'd love your feedback.</t>
+          <t>This two-minute survey will guide our future collaborations and help us recommend the right artists and editions for your collection.</t>
         </is>
       </c>
       <c r="C76" s="10">
-        <f>SUBSTITUTE(B76,"{artist}",Inputs!$B$4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77" ht="32" customHeight="1">
+        <f>B76</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77" ht="48" customHeight="1">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>email · non-purchaser survey · 2</t>
+          <t>email · non-purchaser survey · 3</t>
         </is>
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>This two-minute survey will guide our future collaborations and help us recommend the right artists and editions for your collection.</t>
+          <t>As a thank you for taking part in the survey and helping us improve the collector experience, you'll be entered into a draw to win a €500 Avant Arte gift card.</t>
         </is>
       </c>
       <c r="C77" s="10">
@@ -2442,15 +2464,15 @@
         <v/>
       </c>
     </row>
-    <row r="78" ht="48" customHeight="1">
+    <row r="78" ht="16" customHeight="1">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>email · non-purchaser survey · 3</t>
+          <t>email · non-purchaser survey · terms</t>
         </is>
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>As a thank you for taking part in the survey and helping us improve the collector experience, you'll be entered into a draw to win a €500 Avant Arte gift card.</t>
+          <t>You can read the terms here.</t>
         </is>
       </c>
       <c r="C78" s="10">
@@ -2461,12 +2483,12 @@
     <row r="79" ht="16" customHeight="1">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>email · non-purchaser survey · terms</t>
+          <t>email · non-purchaser survey · footer</t>
         </is>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>You can read the terms here.</t>
+          <t>What can we do better?</t>
         </is>
       </c>
       <c r="C79" s="10">
@@ -2474,74 +2496,58 @@
         <v/>
       </c>
     </row>
-    <row r="80" ht="16" customHeight="1">
-      <c r="A80" s="4" t="inlineStr">
-        <is>
-          <t>email · non-purchaser survey · footer</t>
-        </is>
-      </c>
-      <c r="B80" s="8" t="inlineStr">
-        <is>
-          <t>What can we do better?</t>
-        </is>
-      </c>
-      <c r="C80" s="10">
-        <f>B80</f>
-        <v/>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="3" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
         <is>
           <t>EMAILS · monthly preview</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="16" customHeight="1">
+    <row r="81" ht="16" customHeight="1">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>email · monthly preview · opener</t>
+        </is>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>From {artist} comes {work_intro}{support}.</t>
+        </is>
+      </c>
+      <c r="C81" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B81,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$38),"{support}",Inputs!$B$39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82" ht="32" customHeight="1">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>email · monthly preview · opener</t>
+          <t>email · monthly preview · when, draw</t>
         </is>
       </c>
       <c r="B82" s="8" t="inlineStr">
         <is>
-          <t>From {artist} comes {work_intro}{support}.</t>
+          <t>The edition will be allocated by a randomised draw, which closes at {close_time} on {close_date}.</t>
         </is>
       </c>
       <c r="C82" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B82,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$38),"{support}",Inputs!$B$39)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B82,"{close_date}",Inputs!$B$52),"{close_time}",Inputs!$B$53)</f>
         <v/>
       </c>
     </row>
     <row r="83" ht="32" customHeight="1">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>email · monthly preview · when, draw</t>
+          <t>email · monthly preview · when, timed</t>
         </is>
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>The edition will be allocated by a randomised draw, which closes at {close_time} on {close_date}.</t>
+          <t>The edition will be available to collect for {window} only, from {launch_time} on {launch_weekday}, {launch_date_dd}.</t>
         </is>
       </c>
       <c r="C83" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B83,"{close_date}",Inputs!$B$53),"{close_time}",Inputs!$B$54)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84" ht="32" customHeight="1">
-      <c r="A84" s="4" t="inlineStr">
-        <is>
-          <t>email · monthly preview · when, timed</t>
-        </is>
-      </c>
-      <c r="B84" s="8" t="inlineStr">
-        <is>
-          <t>The edition will be available to collect for {window} only, from {launch_time} on {launch_weekday}, {launch_date_dd}.</t>
-        </is>
-      </c>
-      <c r="C84" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B84,"{window}",Inputs!$B$13),"{launch_time}",Inputs!$B$50),"{launch_weekday}",Inputs!$B$51),"{launch_date_dd}",Inputs!$B$52)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B83,"{window}",Inputs!$B$13),"{launch_time}",Inputs!$B$49),"{launch_weekday}",Inputs!$B$50),"{launch_date_dd}",Inputs!$B$51)</f>
         <v/>
       </c>
     </row>
@@ -2703,7 +2709,7 @@
         <v/>
       </c>
       <c r="F5" s="11">
-        <f>Lines!$C$15&amp;IF(Inputs!$B$43,"",IF(Inputs!$B$40="",""," "&amp;Lines!$C$16))</f>
+        <f>Lines!$C$15&amp;IF(Inputs!$B$42,"",IF(Inputs!$B$40="",""," "&amp;Lines!$C$16))</f>
         <v/>
       </c>
       <c r="G5" s="11">
@@ -2742,7 +2748,7 @@
         <v/>
       </c>
       <c r="E6" s="11">
-        <f>Inputs!$B$48</f>
+        <f>Inputs!$B$47</f>
         <v/>
       </c>
       <c r="F6" s="11">
@@ -3083,11 +3089,11 @@
         <v/>
       </c>
       <c r="F4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$12="draw","Enter the draw for a chance to collect. Closes "&amp;Inputs!$B$53&amp;".","Launching "&amp;Inputs!$B$49&amp;". Register for updates."))</f>
+        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$12="draw","Enter the draw for a chance to collect. Closes "&amp;Inputs!$B$52&amp;".","Launching "&amp;Inputs!$B$48&amp;". Register for updates."))</f>
         <v/>
       </c>
       <c r="G4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$12="draw","Enter the draw","Launching "&amp;Inputs!$B$49))</f>
+        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$12="draw","Enter the draw","Launching "&amp;Inputs!$B$48))</f>
         <v/>
       </c>
       <c r="H4" s="11">
@@ -3095,7 +3101,7 @@
         <v/>
       </c>
       <c r="I4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",(Lines!$C$30&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$47&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$45&amp;CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$12="draw",Lines!$C$26,(Lines!$C$31&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$32))))</f>
+        <f>IF($D4&lt;&gt;"yes","",(Lines!$C$30&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$46&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$44&amp;CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$12="draw",Lines!$C$26,(Lines!$C$31&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$32))))</f>
         <v/>
       </c>
       <c r="J4" s="11">
@@ -3103,15 +3109,15 @@
         <v/>
       </c>
       <c r="K4" s="11">
+        <f>IF($D4&lt;&gt;"yes","",Inputs!$B$60)</f>
+        <v/>
+      </c>
+      <c r="L4" s="11">
         <f>IF($D4&lt;&gt;"yes","",Inputs!$B$61)</f>
         <v/>
       </c>
-      <c r="L4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",Inputs!$B$62)</f>
-        <v/>
-      </c>
       <c r="M4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$12="draw","Collect "&amp;Inputs!$B$57,"Launching "&amp;Inputs!$B$49))</f>
+        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$12="draw","Collect "&amp;Inputs!$B$56,"Launching "&amp;Inputs!$B$48))</f>
         <v/>
       </c>
       <c r="N4" s="11">
@@ -3158,7 +3164,7 @@
         <v/>
       </c>
       <c r="I5" s="11">
-        <f>IF($D5&lt;&gt;"yes","",(Lines!$C$34&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$35&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$36&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$37&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$38))</f>
+        <f>IF($D5&lt;&gt;"yes","",(Lines!$C$34&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$35&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$36&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$37))</f>
         <v/>
       </c>
       <c r="J5" s="11">
@@ -3221,7 +3227,7 @@
         <v/>
       </c>
       <c r="I6" s="11">
-        <f>IF($D6&lt;&gt;"yes","",(Lines!$C$24&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$40&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$46&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$41&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$43))</f>
+        <f>IF($D6&lt;&gt;"yes","",(Lines!$C$24&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$39&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$45&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$40&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$42))</f>
         <v/>
       </c>
       <c r="J6" s="11">
@@ -3284,7 +3290,7 @@
         <v/>
       </c>
       <c r="I7" s="11">
-        <f>IF($D7&lt;&gt;"yes","",(Lines!$C$24&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$40&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$46&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$42&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$43&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$27&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$25))</f>
+        <f>IF($D7&lt;&gt;"yes","",(Lines!$C$24&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$39&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$45&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$41&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$42&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$27&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$25))</f>
         <v/>
       </c>
       <c r="J7" s="11">
@@ -3292,7 +3298,7 @@
         <v/>
       </c>
       <c r="K7" s="11">
-        <f>IF($D7&lt;&gt;"yes","",Inputs!$B$61)</f>
+        <f>IF($D7&lt;&gt;"yes","",Inputs!$B$60)</f>
         <v/>
       </c>
       <c r="L7" s="11">
@@ -3347,7 +3353,7 @@
         <v/>
       </c>
       <c r="I8" s="11">
-        <f>IF($D8&lt;&gt;"yes","",(Lines!$C$24&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$47&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$12="draw",Lines!$C$48,Lines!$C$49)&amp;CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$12="draw",Lines!$C$50,Lines!$C$51)&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$25&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$52))</f>
+        <f>IF($D8&lt;&gt;"yes","",(Lines!$C$24&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$46&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$12="draw",Lines!$C$47,Lines!$C$48)&amp;CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$12="draw",Lines!$C$49,Lines!$C$50)&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$25&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$51))</f>
         <v/>
       </c>
       <c r="J8" s="11">
@@ -3355,7 +3361,7 @@
         <v/>
       </c>
       <c r="K8" s="11">
-        <f>IF($D8&lt;&gt;"yes","",Inputs!$B$61)</f>
+        <f>IF($D8&lt;&gt;"yes","",Inputs!$B$60)</f>
         <v/>
       </c>
       <c r="L8" s="11">
@@ -3410,7 +3416,7 @@
         <v/>
       </c>
       <c r="I9" s="11">
-        <f>IF($D9&lt;&gt;"yes","",(Lines!$C$24&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$44&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$45&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$46&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$27&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$25))</f>
+        <f>IF($D9&lt;&gt;"yes","",(Lines!$C$24&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$43&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$44&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$45&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$27&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$25))</f>
         <v/>
       </c>
       <c r="J9" s="11">
@@ -3418,7 +3424,7 @@
         <v/>
       </c>
       <c r="K9" s="11">
-        <f>IF($D9&lt;&gt;"yes","",Inputs!$B$61)</f>
+        <f>IF($D9&lt;&gt;"yes","",Inputs!$B$60)</f>
         <v/>
       </c>
       <c r="L9" s="11">
@@ -3461,7 +3467,7 @@
         <v/>
       </c>
       <c r="F10" s="11">
-        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$59&amp;", starting now.")</f>
+        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$58&amp;", starting now.")</f>
         <v/>
       </c>
       <c r="G10" s="11">
@@ -3469,11 +3475,11 @@
         <v/>
       </c>
       <c r="H10" s="11">
-        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$59&amp;", starting now")</f>
+        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$58&amp;", starting now")</f>
         <v/>
       </c>
       <c r="I10" s="11">
-        <f>IF($D10&lt;&gt;"yes","",(Lines!$C$54&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$47&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$46&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$55))</f>
+        <f>IF($D10&lt;&gt;"yes","",(Lines!$C$53&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$46&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$45&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$54))</f>
         <v/>
       </c>
       <c r="J10" s="11">
@@ -3481,15 +3487,15 @@
         <v/>
       </c>
       <c r="K10" s="11">
+        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$60)</f>
+        <v/>
+      </c>
+      <c r="L10" s="11">
         <f>IF($D10&lt;&gt;"yes","",Inputs!$B$61)</f>
         <v/>
       </c>
-      <c r="L10" s="11">
-        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$62)</f>
-        <v/>
-      </c>
       <c r="M10" s="11">
-        <f>IF($D10&lt;&gt;"yes","","Collect "&amp;Inputs!$B$57)</f>
+        <f>IF($D10&lt;&gt;"yes","","Collect "&amp;Inputs!$B$56)</f>
         <v/>
       </c>
       <c r="N10" s="11">
@@ -3528,11 +3534,11 @@
         <v/>
       </c>
       <c r="G11" s="11">
+        <f>IF($D11&lt;&gt;"yes","",Lines!$C$55)</f>
+        <v/>
+      </c>
+      <c r="H11" s="11">
         <f>IF($D11&lt;&gt;"yes","",Lines!$C$56)</f>
-        <v/>
-      </c>
-      <c r="H11" s="11">
-        <f>IF($D11&lt;&gt;"yes","",Lines!$C$57)</f>
         <v/>
       </c>
       <c r="I11" s="11">
@@ -3552,7 +3558,7 @@
         <v/>
       </c>
       <c r="M11" s="11">
-        <f>IF($D11&lt;&gt;"yes","",Lines!$C$58)</f>
+        <f>IF($D11&lt;&gt;"yes","",Lines!$C$57)</f>
         <v/>
       </c>
       <c r="N11" s="11">
@@ -3591,11 +3597,11 @@
         <v/>
       </c>
       <c r="G12" s="11">
-        <f>IF($D12&lt;&gt;"yes","",Lines!$C$56)</f>
+        <f>IF($D12&lt;&gt;"yes","",Lines!$C$55)</f>
         <v/>
       </c>
       <c r="H12" s="11">
-        <f>IF($D12&lt;&gt;"yes","",Lines!$C$59)</f>
+        <f>IF($D12&lt;&gt;"yes","",Lines!$C$58)</f>
         <v/>
       </c>
       <c r="I12" s="11">
@@ -3615,7 +3621,7 @@
         <v/>
       </c>
       <c r="M12" s="11">
-        <f>IF($D12&lt;&gt;"yes","",Lines!$C$60)</f>
+        <f>IF($D12&lt;&gt;"yes","",Lines!$C$59)</f>
         <v/>
       </c>
       <c r="N12" s="11">
@@ -3658,11 +3664,11 @@
         <v/>
       </c>
       <c r="H13" s="11">
-        <f>IF($D13&lt;&gt;"yes","",Lines!$C$61)</f>
+        <f>IF($D13&lt;&gt;"yes","",Lines!$C$60)</f>
         <v/>
       </c>
       <c r="I13" s="11">
-        <f>IF($D13&lt;&gt;"yes","",(Lines!$C$62&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$63))</f>
+        <f>IF($D13&lt;&gt;"yes","",(Lines!$C$61&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$62))</f>
         <v/>
       </c>
       <c r="J13" s="11">
@@ -3670,7 +3676,7 @@
         <v/>
       </c>
       <c r="K13" s="11">
-        <f>IF($D13&lt;&gt;"yes","",Inputs!$B$61)</f>
+        <f>IF($D13&lt;&gt;"yes","",Inputs!$B$60)</f>
         <v/>
       </c>
       <c r="L13" s="11">
@@ -3678,7 +3684,7 @@
         <v/>
       </c>
       <c r="M13" s="11">
-        <f>IF($D13&lt;&gt;"yes","",Lines!$C$64)</f>
+        <f>IF($D13&lt;&gt;"yes","",Lines!$C$63)</f>
         <v/>
       </c>
       <c r="N13" s="11">
@@ -3713,7 +3719,7 @@
         <v/>
       </c>
       <c r="F14" s="11">
-        <f>IF($D14&lt;&gt;"yes","",IF(Inputs!$B$12="draw","The draw closes at "&amp;Inputs!$B$54&amp;" on "&amp;Inputs!$B$53&amp;".","Time is almost up."))</f>
+        <f>IF($D14&lt;&gt;"yes","",IF(Inputs!$B$12="draw","The draw closes at "&amp;Inputs!$B$53&amp;" on "&amp;Inputs!$B$52&amp;".","Time is almost up."))</f>
         <v/>
       </c>
       <c r="G14" s="11">
@@ -3725,7 +3731,7 @@
         <v/>
       </c>
       <c r="I14" s="11">
-        <f>IF($D14&lt;&gt;"yes","",IF(Inputs!$B$12="draw",(Lines!$C$68&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$69),(Lines!$C$66&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$67)))</f>
+        <f>IF($D14&lt;&gt;"yes","",IF(Inputs!$B$12="draw",(Lines!$C$67&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$68),(Lines!$C$65&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$66)))</f>
         <v/>
       </c>
       <c r="J14" s="11">
@@ -3733,7 +3739,7 @@
         <v/>
       </c>
       <c r="K14" s="11">
-        <f>IF($D14&lt;&gt;"yes","",Inputs!$B$61)</f>
+        <f>IF($D14&lt;&gt;"yes","",Inputs!$B$60)</f>
         <v/>
       </c>
       <c r="L14" s="11">
@@ -3772,7 +3778,7 @@
         <v/>
       </c>
       <c r="E15" s="11">
-        <f>IF($D15&lt;&gt;"yes","",Lines!$C$71)</f>
+        <f>IF($D15&lt;&gt;"yes","",Lines!$C$70)</f>
         <v/>
       </c>
       <c r="F15" s="11">
@@ -3788,7 +3794,7 @@
         <v/>
       </c>
       <c r="I15" s="11">
-        <f>IF($D15&lt;&gt;"yes","",(Lines!$C$24&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$72&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$73&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$74&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$75))</f>
+        <f>IF($D15&lt;&gt;"yes","",(Lines!$C$24&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$71&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$72&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$73&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$74))</f>
         <v/>
       </c>
       <c r="J15" s="11">
@@ -3851,7 +3857,7 @@
         <v/>
       </c>
       <c r="I16" s="11">
-        <f>IF($D16&lt;&gt;"yes","",(Lines!$C$76&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$77&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$78&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$79))</f>
+        <f>IF($D16&lt;&gt;"yes","",(Lines!$C$75&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$76&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$77&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$78))</f>
         <v/>
       </c>
       <c r="J16" s="11">
@@ -3867,7 +3873,7 @@
         <v/>
       </c>
       <c r="M16" s="11">
-        <f>IF($D16&lt;&gt;"yes","",Lines!$C$80)</f>
+        <f>IF($D16&lt;&gt;"yes","",Lines!$C$79)</f>
         <v/>
       </c>
       <c r="N16" s="11">
@@ -3914,7 +3920,7 @@
         <v/>
       </c>
       <c r="I17" s="11">
-        <f>IF($D17&lt;&gt;"yes","",(Lines!$C$82&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$47&amp;CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$12="draw",Lines!$C$83,Lines!$C$84)))</f>
+        <f>IF($D17&lt;&gt;"yes","",(Lines!$C$81&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$46&amp;CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$12="draw",Lines!$C$82,Lines!$C$83)))</f>
         <v/>
       </c>
       <c r="J17" s="11">

</xml_diff>

<commit_message>
Add the Insiders channel tag and the Twitter set
The Insiders account posts the same caption as the main feed (the archive
shows them near-identical for the same campaigns), so the Posts sheet and the
Instagram template carry a channel tag per post instead of new lines:
Announcement, Now Live and Halfway for a timed edition, Announcement for a draw.

Tweets are the post's status line with the X handle, the hook on the
announcement only, the beneficiary named once, and an action line that ends
with the release's link: sign up for updates, enter the draw, or buy a print.
No features line, no hashtag, no bio. Six new lines; the status lines are
reused with the X handle swapped in. New Tweets sheet in the workbook, a
twitter-set template, two brief fields (x_handle, link), and a tweet check in
the validator that flags "link in bio" and warns over 280 characters.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KCpXfXvgVaMZkSdhMYLgwy
</commit_message>
<xml_diff>
--- a/tool/release-copy.xlsx
+++ b/tool/release-copy.xlsx
@@ -10,8 +10,9 @@
     <sheet name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Lines" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Posts" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Emails" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Rules" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Tweets" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Emails" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Rules" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -491,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -567,736 +568,777 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>hashtag</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>GraysonPerry</t>
-        </is>
-      </c>
+          <t>x_handle</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr"/>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>announcement post only; blank for none</t>
+          <t>X (Twitter) handle, blank if none</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>ordinal</t>
+          <t>link</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>latest</t>
+          <t>https://avantarte.co/grayson-perry</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>debut, latest or second</t>
+          <t>the release's short link, for tweets</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>hashtag</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>The Changeling</t>
+          <t>GraysonPerry</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>exactly as it appears; for a series with one shared title, give the series name</t>
+          <t>announcement post only; blank for none</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>is_series</t>
+          <t>ordinal</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>latest</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>yes when the works share one title</t>
+          <t>debut, latest or second</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>edition_phrase</t>
+          <t>title</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>a new limited edition print</t>
+          <t>The Changeling</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>e.g. a trio of limited edition prints; six new limited edition prints</t>
+          <t>exactly as it appears; for a series with one shared title, give the series name</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>works</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>1</v>
+          <t>is_series</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>number of works</t>
+          <t>yes when the works share one title</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>mechanic</t>
+          <t>edition_phrase</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>timed</t>
+          <t>a new limited edition print</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>timed (TL) or draw (LE)</t>
+          <t>e.g. a trio of limited edition prints; six new limited edition prints</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>window</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>one week</t>
-        </is>
+          <t>works</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>1</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>48 hours or one week; timed only</t>
+          <t>number of works</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>launch_at</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="n">
-        <v>46142.58333333334</v>
+          <t>mechanic</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>timed</t>
+        </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>date and time the window opens, or the draw opens (UK)</t>
+          <t>timed (TL) or draw (LE)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>closes_at</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="n">
-        <v>46149.58333333334</v>
+          <t>window</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>one week</t>
+        </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>date and time the window or draw closes (UK)</t>
+          <t>48 hours or one week; timed only</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>beneficiary</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>the Foundling Museum</t>
-        </is>
+          <t>launch_at</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>46142.58333333334</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>as it reads mid-sentence; blank if none</t>
+          <t>date and time the window opens, or the draw opens (UK)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>beneficiary_handle</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>foundlingmuseum</t>
-        </is>
+          <t>closes_at</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>46149.58333333334</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>blank if none</t>
+          <t>date and time the window or draw closes (UK)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>advisor</t>
+          <t>beneficiary</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Sam</t>
+          <t>the Foundling Museum</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>signs the Insiders email and the first-time collector survey: Sofiya, Curtis or Sam</t>
+          <t>as it reads mid-sentence; blank if none</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>early_access_code</t>
+          <t>beneficiary_handle</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>000-000</t>
+          <t>foundlingmuseum</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>draw releases</t>
+          <t>blank if none</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>feature_1</t>
+          <t>advisor</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Signed by the artist</t>
+          <t>Sam</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>the standard three; clear a cell to drop it</t>
+          <t>signs the Insiders email and the first-time collector survey: Sofiya, Curtis or Sam</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>feature_2</t>
+          <t>early_access_code</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Individually numbered</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr"/>
+          <t>000-000</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>draw releases</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>feature_3</t>
+          <t>feature_1</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Free worldwide shipping</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr"/>
+          <t>Signed by the artist</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>the standard three; clear a cell to drop it</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>feature_4</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr"/>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>bespoke, e.g. Hand-finished by the artist. Never 'our'.</t>
-        </is>
-      </c>
+          <t>feature_2</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Individually numbered</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
+          <t>feature_3</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Free worldwide shipping</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>feature_4</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr"/>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>bespoke, e.g. Hand-finished by the artist. Never 'our'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
           <t>feature_5</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr"/>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr"/>
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>bespoke, e.g. Available individually or as a set</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>Fragments, written once per release. Voice-neutral: no we or our, no artist name in the hook or making line.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="128" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="29" ht="128" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>bio</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>Grayson Perry has long been one of the most distinctive voices in contemporary British art.
 Working across ceramics, tapestry, print and sculpture, his practice examines identity, class, and gender in modern society. Drawing on autobiography as well as social observation, Grayson often pairs the decorative language of traditional craft with direct commentary on the structures and contradictions that shape everyday life.</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C29" s="9" t="inlineStr">
         <is>
           <t>2 to 3 sentences on the artist, third person, no handle. Coming Soon post only.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="48" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="30" ht="48" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>hook</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>The Changeling portrays a child as a symbol of modern youth, exploring how technology shapes today's generations. It reimagines changeling folklore for the digital age, and is intended to be 'quite disturbing'.</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>1 to 2 sentences about the work only. Reused in every post and email.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="32" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>making</t>
         </is>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>To create the edition, printmakers at Make-Ready translated a new design into a 9-colour silkscreen, capturing the vivid detail of the original drawing.</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr">
+      <c r="C31" s="9" t="inlineStr">
         <is>
           <t>one sentence, written as 'printmakers at Make-Ready'; the sheet adds 'our'.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="32" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>quote</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>Beauty and seriousness are perhaps the most shocking tactics left to artists these days.</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>verbatim, a complete sentence, or blank</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="7" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
         <is>
           <t>Derived (formulas, do not edit)</t>
         </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>named</t>
-        </is>
-      </c>
-      <c r="B33" s="10">
-        <f>$B$4&amp;IF($B$5="",""," (@"&amp;$B$5&amp;")")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>work</t>
-        </is>
-      </c>
-      <c r="B34" s="10">
-        <f>IF($B$9="yes","the "&amp;$B$8&amp;" series","‘"&amp;$B$8&amp;"’")</f>
-        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Work</t>
+          <t>named</t>
         </is>
       </c>
       <c r="B35" s="10">
-        <f>UPPER(LEFT($B$34,1))&amp;MID($B$34,2,999)</f>
+        <f>$B$4&amp;IF($B$5="",""," (@"&amp;$B$5&amp;")")</f>
         <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>work_email</t>
+          <t>named_x</t>
         </is>
       </c>
       <c r="B36" s="10">
-        <f>IF($B$9="yes","the "&amp;$B$8&amp;" series",$B$8)</f>
+        <f>$B$4&amp;IF($B$6="",""," (@"&amp;$B$6&amp;")")</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Work_email</t>
+          <t>work</t>
         </is>
       </c>
       <c r="B37" s="10">
-        <f>UPPER(LEFT($B$36,1))&amp;MID($B$36,2,999)</f>
+        <f>IF($B$11="yes","the "&amp;$B$10&amp;" series","‘"&amp;$B$10&amp;"’")</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>work_intro</t>
+          <t>Work</t>
         </is>
       </c>
       <c r="B38" s="10">
-        <f>IF($B$9="yes",$B$10&amp;" from the "&amp;$B$8&amp;" series",IF($B$11=1,$B$8&amp;", "&amp;$B$10,$B$10))</f>
+        <f>UPPER(LEFT($B$37,1))&amp;MID($B$37,2,999)</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>support</t>
+          <t>work_email</t>
         </is>
       </c>
       <c r="B39" s="10">
-        <f>IF(OR($B$16="",$B$42),"",", released in support of "&amp;$B$16)</f>
+        <f>IF($B$11="yes","the "&amp;$B$10&amp;" series",$B$10)</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>beneficiary_tagged</t>
+          <t>Work_email</t>
         </is>
       </c>
       <c r="B40" s="10">
-        <f>IF($B$16="","",$B$16&amp;IF($B$17="",""," (@"&amp;$B$17&amp;")"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" ht="80" customHeight="1">
+        <f>UPPER(LEFT($B$39,1))&amp;MID($B$39,2,999)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>bio_tagged</t>
+          <t>work_intro</t>
         </is>
       </c>
       <c r="B41" s="10">
-        <f>IF($B$5="",$B$27,SUBSTITUTE($B$27,$B$4,$B$33,1))</f>
+        <f>IF($B$11="yes",$B$12&amp;" from the "&amp;$B$10&amp;" series",IF($B$13=1,$B$10&amp;", "&amp;$B$12,$B$12))</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>hook_names_beneficiary</t>
+          <t>support</t>
         </is>
       </c>
       <c r="B42" s="10">
-        <f>IF($B$16="",FALSE,ISNUMBER(SEARCH($B$16,$B$28)))</f>
+        <f>IF(OR($B$18="",$B$45),"",", released in support of "&amp;$B$18)</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>features</t>
+          <t>beneficiary_tagged</t>
         </is>
       </c>
       <c r="B43" s="10">
-        <f>$B$20&amp;IF($B$21="","",". "&amp;$B$21)&amp;IF($B$22="","",". "&amp;$B$22)&amp;IF($B$23="","",". "&amp;$B$23)&amp;IF($B$24="","",". "&amp;$B$24)&amp;"."</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" ht="60" customHeight="1">
+        <f>IF($B$18="","",$B$18&amp;IF($B$19="",""," (@"&amp;$B$19&amp;")"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="80" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>features_list</t>
+          <t>bio_tagged</t>
         </is>
       </c>
       <c r="B44" s="10">
-        <f>"· "&amp;$B$20&amp;IF($B$21="","",CHAR(10)&amp;"· "&amp;$B$21)&amp;IF($B$22="","",CHAR(10)&amp;"· "&amp;$B$22)&amp;IF($B$23="","",CHAR(10)&amp;"· "&amp;$B$23)&amp;IF($B$24="","",CHAR(10)&amp;"· "&amp;$B$24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" ht="70" customHeight="1">
+        <f>IF($B$5="",$B$29,SUBSTITUTE($B$29,$B$4,$B$35,1))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>features_list_support</t>
+          <t>hook_names_beneficiary</t>
         </is>
       </c>
       <c r="B45" s="10">
-        <f>$B$44&amp;IF(OR($B$16="",$B$42),"",CHAR(10)&amp;"· Released in support of "&amp;$B$16)</f>
+        <f>IF($B$18="",FALSE,ISNUMBER(SEARCH($B$18,$B$30)))</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>making_ours</t>
+          <t>features</t>
         </is>
       </c>
       <c r="B46" s="10">
-        <f>SUBSTITUTE($B$29,"printmakers at Make-Ready","our printmakers at Make-Ready")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
+        <f>$B$22&amp;IF($B$23="","",". "&amp;$B$23)&amp;IF($B$24="","",". "&amp;$B$24)&amp;IF($B$25="","",". "&amp;$B$25)&amp;IF($B$26="","",". "&amp;$B$26)&amp;"."</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="60" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>making_ours_tagged</t>
+          <t>features_list</t>
         </is>
       </c>
       <c r="B47" s="10">
-        <f>SUBSTITUTE($B$29,"printmakers at Make-Ready","our printmakers at Make-Ready (@make__ready)")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
+        <f>"· "&amp;$B$22&amp;IF($B$23="","",CHAR(10)&amp;"· "&amp;$B$23)&amp;IF($B$24="","",CHAR(10)&amp;"· "&amp;$B$24)&amp;IF($B$25="","",CHAR(10)&amp;"· "&amp;$B$25)&amp;IF($B$26="","",CHAR(10)&amp;"· "&amp;$B$26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="70" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>launch_date</t>
+          <t>features_list_support</t>
         </is>
       </c>
       <c r="B48" s="10">
-        <f>TEXT($B$14,"d mmmm")</f>
+        <f>$B$47&amp;IF(OR($B$18="",$B$45),"",CHAR(10)&amp;"· Released in support of "&amp;$B$18)</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>launch_time</t>
+          <t>making_ours</t>
         </is>
       </c>
       <c r="B49" s="10">
-        <f>TEXT($B$14,"hh:mm")&amp;" UK time"</f>
+        <f>SUBSTITUTE($B$31,"printmakers at Make-Ready","our printmakers at Make-Ready")</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>launch_weekday</t>
+          <t>making_ours_tagged</t>
         </is>
       </c>
       <c r="B50" s="10">
-        <f>TEXT($B$14,"dddd")</f>
+        <f>SUBSTITUTE($B$31,"printmakers at Make-Ready","our printmakers at Make-Ready (@make__ready)")</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>launch_date_dd</t>
+          <t>launch_date</t>
         </is>
       </c>
       <c r="B51" s="10">
-        <f>TEXT($B$14,"dd mmmm")</f>
+        <f>TEXT($B$16,"d mmmm")</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>close_date</t>
+          <t>launch_time</t>
         </is>
       </c>
       <c r="B52" s="10">
-        <f>TEXT($B$15,"d mmmm")</f>
+        <f>TEXT($B$16,"hh:mm")&amp;" UK time"</f>
         <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>close_time</t>
+          <t>launch_weekday</t>
         </is>
       </c>
       <c r="B53" s="10">
-        <f>TEXT($B$15,"hh:mm")&amp;" UK time"</f>
+        <f>TEXT($B$16,"dddd")</f>
         <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>close_weekday</t>
+          <t>launch_date_dd</t>
         </is>
       </c>
       <c r="B54" s="10">
-        <f>TEXT($B$15,"dddd")</f>
+        <f>TEXT($B$16,"dd mmmm")</f>
         <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>close_date_dd</t>
+          <t>close_date</t>
         </is>
       </c>
       <c r="B55" s="10">
-        <f>TEXT($B$15,"dd mmmm")</f>
+        <f>TEXT($B$17,"d mmmm")</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>collect_phrase</t>
+          <t>close_time</t>
         </is>
       </c>
       <c r="B56" s="10">
-        <f>SUBSTITUTE($B$10," new "," ")</f>
+        <f>TEXT($B$17,"hh:mm")&amp;" UK time"</f>
         <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>edition_phrase_cap</t>
+          <t>close_weekday</t>
         </is>
       </c>
       <c r="B57" s="10">
-        <f>UPPER(LEFT($B$10,1))&amp;MID($B$10,2,999)</f>
+        <f>TEXT($B$17,"dddd")</f>
         <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>window_cap</t>
+          <t>close_date_dd</t>
         </is>
       </c>
       <c r="B58" s="10">
-        <f>UPPER(LEFT($B$13,1))&amp;MID($B$13,2,999)</f>
+        <f>TEXT($B$17,"dd mmmm")</f>
         <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>card_line</t>
+          <t>collect_phrase</t>
         </is>
       </c>
       <c r="B59" s="10">
-        <f>$B$57&amp;" by "&amp;$B$4&amp;"."</f>
+        <f>SUBSTITUTE($B$12," new "," ")</f>
         <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>card</t>
+          <t>edition_phrase_cap</t>
         </is>
       </c>
       <c r="B60" s="10">
-        <f>$B$8&amp;CHAR(10)&amp;$B$59</f>
+        <f>UPPER(LEFT($B$12,1))&amp;MID($B$12,2,999)</f>
         <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>quote_line</t>
+          <t>window_cap</t>
         </is>
       </c>
       <c r="B61" s="10">
-        <f>IF($B$30="","","“"&amp;$B$30&amp;"” – "&amp;$B$4)</f>
+        <f>UPPER(LEFT($B$15,1))&amp;MID($B$15,2,999)</f>
         <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>each_artwork</t>
+          <t>card_line</t>
         </is>
       </c>
       <c r="B62" s="10">
-        <f>IF($B$11&gt;1," for each artwork","")</f>
+        <f>$B$60&amp;" by "&amp;$B$4&amp;"."</f>
         <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>work_word</t>
+          <t>card</t>
         </is>
       </c>
       <c r="B63" s="10">
-        <f>IF($B$11&gt;1,"works","work")</f>
+        <f>$B$10&amp;CHAR(10)&amp;$B$62</f>
         <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
+          <t>quote_line</t>
+        </is>
+      </c>
+      <c r="B64" s="10">
+        <f>IF($B$32="","","“"&amp;$B$32&amp;"” – "&amp;$B$4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>each_artwork</t>
+        </is>
+      </c>
+      <c r="B65" s="10">
+        <f>IF($B$13&gt;1," for each artwork","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>work_word</t>
+        </is>
+      </c>
+      <c r="B66" s="10">
+        <f>IF($B$13&gt;1,"works","work")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
           <t>add_what</t>
         </is>
       </c>
-      <c r="B64" s="10">
-        <f>IF($B$11&gt;1,"a print",$B$36)</f>
+      <c r="B67" s="10">
+        <f>IF($B$13&gt;1,"a print",$B$39)</f>
         <v/>
       </c>
     </row>
@@ -1311,7 +1353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1369,7 +1411,7 @@
         </is>
       </c>
       <c r="C5" s="10">
-        <f>SUBSTITUTE(B5,"{ordinal}",Inputs!$B$7)</f>
+        <f>SUBSTITUTE(B5,"{ordinal}",Inputs!$B$9)</f>
         <v/>
       </c>
     </row>
@@ -1385,7 +1427,7 @@
         </is>
       </c>
       <c r="C6" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6,"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{edition_phrase}",Inputs!$B$10)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B6,"{named}",Inputs!$B$35),"{work}",Inputs!$B$37),"{edition_phrase}",Inputs!$B$12)</f>
         <v/>
       </c>
     </row>
@@ -1401,7 +1443,7 @@
         </is>
       </c>
       <c r="C7" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7,"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{edition_phrase}",Inputs!$B$10)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B7,"{named}",Inputs!$B$35),"{work}",Inputs!$B$37),"{edition_phrase}",Inputs!$B$12)</f>
         <v/>
       </c>
     </row>
@@ -1417,7 +1459,7 @@
         </is>
       </c>
       <c r="C8" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8,"{named}",Inputs!$B$33),"{work}",Inputs!$B$34),"{edition_phrase}",Inputs!$B$10)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B8,"{named}",Inputs!$B$35),"{work}",Inputs!$B$37),"{edition_phrase}",Inputs!$B$12)</f>
         <v/>
       </c>
     </row>
@@ -1433,7 +1475,7 @@
         </is>
       </c>
       <c r="C9" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B9,"{artist}",Inputs!$B$4),"{quote}",Inputs!$B$30)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B9,"{artist}",Inputs!$B$4),"{quote}",Inputs!$B$32)</f>
         <v/>
       </c>
     </row>
@@ -1449,7 +1491,7 @@
         </is>
       </c>
       <c r="C10" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B10,"{named}",Inputs!$B$33),"{Work}",Inputs!$B$35),"{edition_phrase}",Inputs!$B$10)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B10,"{named}",Inputs!$B$35),"{Work}",Inputs!$B$38),"{edition_phrase}",Inputs!$B$12)</f>
         <v/>
       </c>
     </row>
@@ -1465,7 +1507,7 @@
         </is>
       </c>
       <c r="C11" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B11,"{named}",Inputs!$B$33),"{Work}",Inputs!$B$35),"{window}",Inputs!$B$13)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B11,"{named}",Inputs!$B$35),"{Work}",Inputs!$B$38),"{window}",Inputs!$B$15)</f>
         <v/>
       </c>
     </row>
@@ -1481,7 +1523,7 @@
         </is>
       </c>
       <c r="C12" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B12,"{named}",Inputs!$B$33),"{work}",Inputs!$B$34)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B12,"{named}",Inputs!$B$35),"{work}",Inputs!$B$37)</f>
         <v/>
       </c>
     </row>
@@ -1497,7 +1539,7 @@
         </is>
       </c>
       <c r="C13" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B13,"{named}",Inputs!$B$33),"{work}",Inputs!$B$34)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B13,"{named}",Inputs!$B$35),"{work}",Inputs!$B$37)</f>
         <v/>
       </c>
     </row>
@@ -1513,7 +1555,7 @@
         </is>
       </c>
       <c r="C14" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B14,"{named}",Inputs!$B$33),"{work}",Inputs!$B$34)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B14,"{named}",Inputs!$B$35),"{work}",Inputs!$B$37)</f>
         <v/>
       </c>
     </row>
@@ -1529,7 +1571,7 @@
         </is>
       </c>
       <c r="C15" s="10">
-        <f>SUBSTITUTE(B15,"{features}",Inputs!$B$43)</f>
+        <f>SUBSTITUTE(B15,"{features}",Inputs!$B$46)</f>
         <v/>
       </c>
     </row>
@@ -1545,7 +1587,7 @@
         </is>
       </c>
       <c r="C16" s="10">
-        <f>SUBSTITUTE(B16,"{beneficiary_tagged}",Inputs!$B$40)</f>
+        <f>SUBSTITUTE(B16,"{beneficiary_tagged}",Inputs!$B$43)</f>
         <v/>
       </c>
     </row>
@@ -1561,7 +1603,7 @@
         </is>
       </c>
       <c r="C17" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17,"{window}",Inputs!$B$13),"{launch_date}",Inputs!$B$48),"{launch_time}",Inputs!$B$49)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B17,"{window}",Inputs!$B$15),"{launch_date}",Inputs!$B$51),"{launch_time}",Inputs!$B$52)</f>
         <v/>
       </c>
     </row>
@@ -1577,7 +1619,7 @@
         </is>
       </c>
       <c r="C18" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B18,"{close_date}",Inputs!$B$52),"{close_time}",Inputs!$B$53)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B18,"{close_date}",Inputs!$B$55),"{close_time}",Inputs!$B$56)</f>
         <v/>
       </c>
     </row>
@@ -1593,7 +1635,7 @@
         </is>
       </c>
       <c r="C19" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B19,"{close_date}",Inputs!$B$52),"{close_time}",Inputs!$B$53)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B19,"{close_date}",Inputs!$B$55),"{close_time}",Inputs!$B$56)</f>
         <v/>
       </c>
     </row>
@@ -1609,7 +1651,7 @@
         </is>
       </c>
       <c r="C20" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B20,"{close_date}",Inputs!$B$52),"{close_time}",Inputs!$B$53)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B20,"{close_date}",Inputs!$B$55),"{close_time}",Inputs!$B$56)</f>
         <v/>
       </c>
     </row>
@@ -1641,145 +1683,145 @@
         </is>
       </c>
       <c r="C22" s="10">
-        <f>SUBSTITUTE(B22,"{hashtag}",Inputs!$B$6)</f>
+        <f>SUBSTITUTE(B22,"{hashtag}",Inputs!$B$8)</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>EMAILS · shared</t>
+          <t>TWEETS</t>
         </is>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>email · greeting</t>
+          <t>tweet · coming soon · status</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Hi {{ personalization_token('contact.firstname', 'there') }},</t>
+          <t>Our {ordinal} collaboration with {named_x} is on the horizon.</t>
         </is>
       </c>
       <c r="C24" s="10">
-        <f>B24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" ht="32" customHeight="1">
+        <f>SUBSTITUTE(SUBSTITUTE(B24,"{named_x}",Inputs!$B$36),"{ordinal}",Inputs!$B$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>email · questions line</t>
+          <t>tweet · coming soon · action</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>If you have any questions, please don't hesitate to get in touch by replying to this email.</t>
+          <t>Sign up for updates: {link}</t>
         </is>
       </c>
       <c r="C25" s="10">
-        <f>B25</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" ht="32" customHeight="1">
+        <f>SUBSTITUTE(B25,"{link}",Inputs!$B$7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>email · draw line</t>
+          <t>tweet · beneficiary line</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Enter the draw for a chance to collect. Closes at {close_time} on {close_date}.</t>
+          <t>Released in support of {beneficiary}.</t>
         </is>
       </c>
       <c r="C26" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B26,"{close_date}",Inputs!$B$52),"{close_time}",Inputs!$B$53)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="64" customHeight="1">
+        <f>SUBSTITUTE(B26,"{beneficiary}",Inputs!$B$18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>email · edition numbers line</t>
+          <t>tweet · action before launch, timed</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Earlier orders will typically receive a lower edition number, with framed editions receiving lower edition numbers than unframed prints. You can read more on how we allocate edition numbers across a release here.</t>
+          <t>Available for {window} from {launch_time} on {launch_date}. Sign up for updates: {link}</t>
         </is>
       </c>
       <c r="C27" s="10">
-        <f>B27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>EMAILS · announcement</t>
-        </is>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B27,"{link}",Inputs!$B$7),"{window}",Inputs!$B$15),"{launch_date}",Inputs!$B$51),"{launch_time}",Inputs!$B$52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>tweet · action, draw</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>Closes {close_date} at {close_time}. Enter the draw: {link}</t>
+        </is>
+      </c>
+      <c r="C28" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B28,"{link}",Inputs!$B$7),"{close_date}",Inputs!$B$55),"{close_time}",Inputs!$B$56)</f>
+        <v/>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>email · announce · subject</t>
+          <t>tweet · action while open, timed</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>{artist} – {edition_phrase_cap}</t>
+          <t>Closes {close_date} at {close_time}. Buy a print: {link}</t>
         </is>
       </c>
       <c r="C29" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B29,"{artist}",Inputs!$B$4),"{edition_phrase_cap}",Inputs!$B$57)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="32" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>email · announce · opener</t>
-        </is>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>We're delighted to announce our {ordinal} collaboration with {artist} – {work_intro}{support}.</t>
-        </is>
-      </c>
-      <c r="C30" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B30,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$38),"{support}",Inputs!$B$39),"{ordinal}",Inputs!$B$7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="32" customHeight="1">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B29,"{link}",Inputs!$B$7),"{close_date}",Inputs!$B$55),"{close_time}",Inputs!$B$56)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>EMAILS · shared</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>email · announce · launch line, timed</t>
+          <t>email · greeting</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>The edition will be available to collect for {window} only, starting at {launch_time} on {launch_weekday}, {launch_date_dd}.</t>
+          <t>Hi {{ personalization_token('contact.firstname', 'there') }},</t>
         </is>
       </c>
       <c r="C31" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B31,"{window}",Inputs!$B$13),"{launch_time}",Inputs!$B$49),"{launch_weekday}",Inputs!$B$50),"{launch_date_dd}",Inputs!$B$51)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="16" customHeight="1">
+        <f>B31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="32" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>email · announce · register line</t>
+          <t>email · questions line</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Click below to learn more and register for updates.</t>
+          <t>If you have any questions, please don't hesitate to get in touch by replying to this email.</t>
         </is>
       </c>
       <c r="C32" s="10">
@@ -1787,22 +1829,31 @@
         <v/>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>EMAILS · welcome (TL flow)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="32" customHeight="1">
+    <row r="33" ht="32" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>email · draw line</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Enter the draw for a chance to collect. Closes at {close_time} on {close_date}.</t>
+        </is>
+      </c>
+      <c r="C33" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(B33,"{close_date}",Inputs!$B$55),"{close_time}",Inputs!$B$56)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="64" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>email · welcome · 1</t>
+          <t>email · edition numbers line</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Welcome {{ personalization_token('contact.firstname', 'to Avant Arte') }}!</t>
+          <t>Earlier orders will typically receive a lower edition number, with framed editions receiving lower edition numbers than unframed prints. You can read more on how we allocate edition numbers across a release here.</t>
         </is>
       </c>
       <c r="C34" s="10">
@@ -1810,102 +1861,93 @@
         <v/>
       </c>
     </row>
-    <row r="35" ht="64" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>email · welcome · 2</t>
-        </is>
-      </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>Avant Arte began with a simple mission – to make collecting art more accessible. Since then, we've collaborated with hundreds of inspiring artists, from rising stars to icons like Ai Weiwei, Jenny Holzer, Lee Ufan and Carrie Mae Weems.</t>
-        </is>
-      </c>
-      <c r="C35" s="10">
-        <f>B35</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="64" customHeight="1">
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>EMAILS · announcement</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="16" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>email · welcome · 3</t>
+          <t>email · announce · subject</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>Our upcoming collaboration with {artist} is the latest in this lineage. If you're new to collecting art or curious about limited editions, our library of guides is a good place to start. In particular, How to collect art and What is an edition?</t>
+          <t>{artist} – {edition_phrase_cap}</t>
         </is>
       </c>
       <c r="C36" s="10">
-        <f>SUBSTITUTE(B36,"{artist}",Inputs!$B$4)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B36,"{artist}",Inputs!$B$4),"{edition_phrase_cap}",Inputs!$B$60)</f>
         <v/>
       </c>
     </row>
     <row r="37" ht="32" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>email · welcome · 4</t>
+          <t>email · announce · opener</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>Let us know if you have any questions. We're excited to see what you collect.</t>
+          <t>We're delighted to announce our {ordinal} collaboration with {artist} – {work_intro}{support}.</t>
         </is>
       </c>
       <c r="C37" s="10">
-        <f>B37</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>EMAILS · early access</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="32" customHeight="1">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B37,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$41),"{support}",Inputs!$B$42),"{ordinal}",Inputs!$B$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="32" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>email · announce · launch line, timed</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>The edition will be available to collect for {window} only, starting at {launch_time} on {launch_weekday}, {launch_date_dd}.</t>
+        </is>
+      </c>
+      <c r="C38" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B38,"{window}",Inputs!$B$15),"{launch_time}",Inputs!$B$52),"{launch_weekday}",Inputs!$B$53),"{launch_date_dd}",Inputs!$B$54)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="16" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>email · early access, timed · opener</t>
+          <t>email · announce · register line</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>Our {ordinal} collaboration with {artist} launches tomorrow at {launch_time} and will be available to collect for {window} only.</t>
+          <t>Click below to learn more and register for updates.</t>
         </is>
       </c>
       <c r="C39" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B39,"{artist}",Inputs!$B$4),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13),"{launch_time}",Inputs!$B$49)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="32" customHeight="1">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>email · early access, timed · registered line</t>
-        </is>
-      </c>
-      <c r="B40" s="8" t="inlineStr">
-        <is>
-          <t>As a thank you for registering for updates, we're offering you the chance to collect the release 24 hours before everyone else.</t>
-        </is>
-      </c>
-      <c r="C40" s="10">
-        <f>B40</f>
-        <v/>
+        <f>B39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>EMAILS · welcome (TL flow)</t>
+        </is>
       </c>
     </row>
     <row r="41" ht="32" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>email · early access, timed · past collectors line</t>
+          <t>email · welcome · 1</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>As a previous collector of the artist, we're offering you the chance to order the collaboration 24 hours before everyone else.</t>
+          <t>Welcome {{ personalization_token('contact.firstname', 'to Avant Arte') }}!</t>
         </is>
       </c>
       <c r="C41" s="10">
@@ -1913,15 +1955,15 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="16" customHeight="1">
+    <row r="42" ht="64" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>email · early access, timed · unlock line</t>
+          <t>email · welcome · 2</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>Unlock early access using the link below.</t>
+          <t>Avant Arte began with a simple mission – to make collecting art more accessible. Since then, we've collaborated with hundreds of inspiring artists, from rising stars to icons like Ai Weiwei, Jenny Holzer, Lee Ufan and Carrie Mae Weems.</t>
         </is>
       </c>
       <c r="C42" s="10">
@@ -1929,328 +1971,319 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="32" customHeight="1">
+    <row r="43" ht="64" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>email · early access, draw · 1</t>
+          <t>email · welcome · 3</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>We're currently preparing the launch of our {ordinal} collaboration with {artist} – {work_intro}{support}.</t>
+          <t>Our upcoming collaboration with {artist} is the latest in this lineage. If you're new to collecting art or curious about limited editions, our library of guides is a good place to start. In particular, How to collect art and What is an edition?</t>
         </is>
       </c>
       <c r="C43" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B43,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$38),"{support}",Inputs!$B$39),"{ordinal}",Inputs!$B$7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" ht="96" customHeight="1">
+        <f>SUBSTITUTE(B43,"{artist}",Inputs!$B$4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="32" customHeight="1">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>email · early access, draw · 2</t>
+          <t>email · welcome · 4</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>The edition will launch publicly on {launch_date} and will be allocated by a randomised draw; however, for the next 48 hours we're offering a small group of collectors a first look, plus access to a limited number of pre-orders. Based on your order history and the artists you've expressed an interest in, I thought the edition would be a good fit for your collection.</t>
+          <t>Let us know if you have any questions. We're excited to see what you collect.</t>
         </is>
       </c>
       <c r="C44" s="10">
-        <f>SUBSTITUTE(B44,"{launch_date}",Inputs!$B$48)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" ht="32" customHeight="1">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>email · early access, draw · 3</t>
-        </is>
-      </c>
-      <c r="B45" s="8" t="inlineStr">
-        <is>
-          <t>Explore the artwork and place your order via the private link below. Use code {early_access_code} to unlock early access.</t>
-        </is>
-      </c>
-      <c r="C45" s="10">
-        <f>SUBSTITUTE(B45,"{early_access_code}",Inputs!$B$19)</f>
-        <v/>
+        <f>B44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>EMAILS · early access</t>
+        </is>
       </c>
     </row>
     <row r="46" ht="32" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
         <is>
+          <t>email · early access, timed · opener</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>Our {ordinal} collaboration with {artist} launches tomorrow at {launch_time} and will be available to collect for {window} only.</t>
+        </is>
+      </c>
+      <c r="C46" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B46,"{artist}",Inputs!$B$4),"{ordinal}",Inputs!$B$9),"{window}",Inputs!$B$15),"{launch_time}",Inputs!$B$52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="32" customHeight="1">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>email · early access, timed · registered line</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>As a thank you for registering for updates, we're offering you the chance to collect the release 24 hours before everyone else.</t>
+        </is>
+      </c>
+      <c r="C47" s="10">
+        <f>B47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="32" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>email · early access, timed · past collectors line</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>As a previous collector of the artist, we're offering you the chance to order the collaboration 24 hours before everyone else.</t>
+        </is>
+      </c>
+      <c r="C48" s="10">
+        <f>B48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>email · early access, timed · unlock line</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>Unlock early access using the link below.</t>
+        </is>
+      </c>
+      <c r="C49" s="10">
+        <f>B49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="32" customHeight="1">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>email · early access, draw · 1</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>We're currently preparing the launch of our {ordinal} collaboration with {artist} – {work_intro}{support}.</t>
+        </is>
+      </c>
+      <c r="C50" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B50,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$41),"{support}",Inputs!$B$42),"{ordinal}",Inputs!$B$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="96" customHeight="1">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>email · early access, draw · 2</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>The edition will launch publicly on {launch_date} and will be allocated by a randomised draw; however, for the next 48 hours we're offering a small group of collectors a first look, plus access to a limited number of pre-orders. Based on your order history and the artists you've expressed an interest in, I thought the edition would be a good fit for your collection.</t>
+        </is>
+      </c>
+      <c r="C51" s="10">
+        <f>SUBSTITUTE(B51,"{launch_date}",Inputs!$B$51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="32" customHeight="1">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>email · early access, draw · 3</t>
+        </is>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>Explore the artwork and place your order via the private link below. Use code {early_access_code} to unlock early access.</t>
+        </is>
+      </c>
+      <c r="C52" s="10">
+        <f>SUBSTITUTE(B52,"{early_access_code}",Inputs!$B$21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" ht="32" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
           <t>email · insiders · opener</t>
         </is>
       </c>
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B53" s="8" t="inlineStr">
         <is>
           <t>I'm delighted to share our {ordinal} collaboration with {artist} – {work_intro}{support}.</t>
         </is>
       </c>
-      <c r="C46" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B46,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$38),"{support}",Inputs!$B$39),"{ordinal}",Inputs!$B$7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" ht="64" customHeight="1">
-      <c r="A47" s="4" t="inlineStr">
+      <c r="C53" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B53,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$41),"{support}",Inputs!$B$42),"{ordinal}",Inputs!$B$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" ht="64" customHeight="1">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>email · insiders · mechanics, draw</t>
         </is>
       </c>
-      <c r="B47" s="8" t="inlineStr">
+      <c r="B54" s="8" t="inlineStr">
         <is>
           <t>The edition will launch publicly on {launch_date} and will be allocated by a randomised draw. However, for the next 48 hours, I'm excited to offer you a first look, plus early access to a limited number of pre-orders.</t>
         </is>
       </c>
-      <c r="C47" s="10">
-        <f>SUBSTITUTE(B47,"{launch_date}",Inputs!$B$48)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" ht="48" customHeight="1">
-      <c r="A48" s="4" t="inlineStr">
+      <c r="C54" s="10">
+        <f>SUBSTITUTE(B54,"{launch_date}",Inputs!$B$51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="48" customHeight="1">
+      <c r="A55" s="4" t="inlineStr">
         <is>
           <t>email · insiders · mechanics, timed</t>
         </is>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B55" s="8" t="inlineStr">
         <is>
           <t>The edition launches tomorrow at {launch_time} and will be available to collect for {window} only. For the next 24 hours, I'm excited to offer you early access ahead of the public launch.</t>
         </is>
       </c>
-      <c r="C48" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B48,"{window}",Inputs!$B$13),"{launch_time}",Inputs!$B$49)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" ht="32" customHeight="1">
-      <c r="A49" s="4" t="inlineStr">
+      <c r="C55" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(B55,"{window}",Inputs!$B$15),"{launch_time}",Inputs!$B$52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" ht="32" customHeight="1">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>email · insiders · code line, draw</t>
         </is>
       </c>
-      <c r="B49" s="8" t="inlineStr">
+      <c r="B56" s="8" t="inlineStr">
         <is>
           <t>Discover the artwork and place your order via the private link below. Use code {early_access_code} to unlock early access.</t>
         </is>
       </c>
-      <c r="C49" s="10">
-        <f>SUBSTITUTE(B49,"{early_access_code}",Inputs!$B$19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" ht="16" customHeight="1">
-      <c r="A50" s="4" t="inlineStr">
+      <c r="C56" s="10">
+        <f>SUBSTITUTE(B56,"{early_access_code}",Inputs!$B$21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" ht="16" customHeight="1">
+      <c r="A57" s="4" t="inlineStr">
         <is>
           <t>email · insiders · link line, timed</t>
         </is>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B57" s="8" t="inlineStr">
         <is>
           <t>Discover the artwork and place your order via the private link below.</t>
         </is>
       </c>
-      <c r="C50" s="10">
-        <f>B50</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" ht="64" customHeight="1">
-      <c r="A51" s="4" t="inlineStr">
+      <c r="C57" s="10">
+        <f>B57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="64" customHeight="1">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>email · insiders · sign-off</t>
         </is>
       </c>
-      <c r="B51" s="8" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>Best regards,
 {advisor}
 Art Advisor at Avant Arte</t>
         </is>
       </c>
-      <c r="C51" s="10">
-        <f>SUBSTITUTE(B51,"{advisor}",Inputs!$B$18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="3" t="inlineStr">
+      <c r="C58" s="10">
+        <f>SUBSTITUTE(B58,"{advisor}",Inputs!$B$20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>EMAILS · the window (TL)</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="32" customHeight="1">
-      <c r="A53" s="4" t="inlineStr">
+    <row r="60" ht="32" customHeight="1">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>email · live · opener</t>
         </is>
       </c>
-      <c r="B53" s="8" t="inlineStr">
+      <c r="B60" s="8" t="inlineStr">
         <is>
           <t>Our {ordinal} collaboration with {artist} is now available to collect for {window} only – {work_intro}{support}.</t>
         </is>
       </c>
-      <c r="C53" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B53,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$38),"{support}",Inputs!$B$39),"{ordinal}",Inputs!$B$7),"{window}",Inputs!$B$13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54" ht="48" customHeight="1">
-      <c r="A54" s="4" t="inlineStr">
+      <c r="C60" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B60,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$41),"{support}",Inputs!$B$42),"{ordinal}",Inputs!$B$9),"{window}",Inputs!$B$15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" ht="48" customHeight="1">
+      <c r="A61" s="4" t="inlineStr">
         <is>
           <t>email · live · closing line</t>
         </is>
       </c>
-      <c r="B54" s="8" t="inlineStr">
+      <c r="B61" s="8" t="inlineStr">
         <is>
           <t>The opportunity to collect an edition ends at {close_time} on {close_weekday}, {close_date_dd}. Click the link below to add {add_what} to your collection.</t>
         </is>
       </c>
-      <c r="C54" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B54,"{close_time}",Inputs!$B$53),"{close_weekday}",Inputs!$B$54),"{close_date_dd}",Inputs!$B$55),"{add_what}",Inputs!$B$64)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55" ht="16" customHeight="1">
-      <c r="A55" s="4" t="inlineStr">
+      <c r="C61" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B61,"{close_time}",Inputs!$B$56),"{close_weekday}",Inputs!$B$57),"{close_date_dd}",Inputs!$B$58),"{add_what}",Inputs!$B$67)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" ht="16" customHeight="1">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>email · halfway · kicker</t>
         </is>
       </c>
-      <c r="B55" s="8" t="inlineStr">
+      <c r="B62" s="8" t="inlineStr">
         <is>
           <t>Collect a print by {artist}</t>
         </is>
       </c>
-      <c r="C55" s="10">
-        <f>SUBSTITUTE(B55,"{artist}",Inputs!$B$4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56" ht="16" customHeight="1">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>email · halfway · headline</t>
-        </is>
-      </c>
-      <c r="B56" s="8" t="inlineStr">
-        <is>
-          <t>24 hours down, 24 to go</t>
-        </is>
-      </c>
-      <c r="C56" s="10">
-        <f>B56</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57" ht="16" customHeight="1">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>email · halfway · footer</t>
-        </is>
-      </c>
-      <c r="B57" s="8" t="inlineStr">
-        <is>
-          <t>There's still time to add a print to your collection.</t>
-        </is>
-      </c>
-      <c r="C57" s="10">
-        <f>B57</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58" ht="16" customHeight="1">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>email · 5 days · headline</t>
-        </is>
-      </c>
-      <c r="B58" s="8" t="inlineStr">
-        <is>
-          <t>2 days down, 5 days to go</t>
-        </is>
-      </c>
-      <c r="C58" s="10">
-        <f>B58</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59" ht="16" customHeight="1">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>email · 5 days · footer</t>
-        </is>
-      </c>
-      <c r="B59" s="8" t="inlineStr">
-        <is>
-          <t>Add a signed print to your collection</t>
-        </is>
-      </c>
-      <c r="C59" s="10">
-        <f>B59</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" ht="16" customHeight="1">
-      <c r="A60" s="4" t="inlineStr">
-        <is>
-          <t>email · 3 days · headline</t>
-        </is>
-      </c>
-      <c r="B60" s="8" t="inlineStr">
-        <is>
-          <t>Three days left to collect</t>
-        </is>
-      </c>
-      <c r="C60" s="10">
-        <f>B60</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61" ht="32" customHeight="1">
-      <c r="A61" s="4" t="inlineStr">
-        <is>
-          <t>email · 3 days · 1</t>
-        </is>
-      </c>
-      <c r="B61" s="8" t="inlineStr">
-        <is>
-          <t>There are just three days left to collect {collect_phrase} by {artist}.</t>
-        </is>
-      </c>
-      <c r="C61" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B61,"{artist}",Inputs!$B$4),"{collect_phrase}",Inputs!$B$56)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62" ht="32" customHeight="1">
-      <c r="A62" s="4" t="inlineStr">
-        <is>
-          <t>email · 3 days · 2</t>
-        </is>
-      </c>
-      <c r="B62" s="8" t="inlineStr">
-        <is>
-          <t>Click the link to collect before {close_time} on {close_weekday}, {close_date_dd}.</t>
-        </is>
-      </c>
       <c r="C62" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B62,"{close_time}",Inputs!$B$53),"{close_weekday}",Inputs!$B$54),"{close_date_dd}",Inputs!$B$55)</f>
+        <f>SUBSTITUTE(B62,"{artist}",Inputs!$B$4)</f>
         <v/>
       </c>
     </row>
     <row r="63" ht="16" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>email · 3 days · footer</t>
+          <t>email · halfway · headline</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>Add a print to your collection</t>
+          <t>24 hours down, 24 to go</t>
         </is>
       </c>
       <c r="C63" s="10">
@@ -2258,93 +2291,111 @@
         <v/>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="3" t="inlineStr">
-        <is>
-          <t>EMAILS · last chance</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="48" customHeight="1">
+    <row r="64" ht="16" customHeight="1">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>email · halfway · footer</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>There's still time to add a print to your collection.</t>
+        </is>
+      </c>
+      <c r="C64" s="10">
+        <f>B64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="16" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>email · last chance, timed · 1</t>
+          <t>email · 5 days · headline</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>It's now or never for our {ordinal} collaboration with {artist} – {collect_phrase} will be available to order until {close_time} on {close_weekday}, {close_date_dd}.</t>
+          <t>2 days down, 5 days to go</t>
         </is>
       </c>
       <c r="C65" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B65,"{artist}",Inputs!$B$4),"{collect_phrase}",Inputs!$B$56),"{ordinal}",Inputs!$B$7),"{close_time}",Inputs!$B$53),"{close_weekday}",Inputs!$B$54),"{close_date_dd}",Inputs!$B$55)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66" ht="32" customHeight="1">
+        <f>B65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" ht="16" customHeight="1">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>email · last chance, timed · 2</t>
+          <t>email · 5 days · footer</t>
         </is>
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>After this time, the edition size{each_artwork} will be confirmed, and the {work_word} will no longer be available to purchase.</t>
+          <t>Add a signed print to your collection</t>
         </is>
       </c>
       <c r="C66" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B66,"{each_artwork}",Inputs!$B$62),"{work_word}",Inputs!$B$63)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67" ht="32" customHeight="1">
+        <f>B66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67" ht="16" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>email · last chance, draw · 1</t>
+          <t>email · 3 days · headline</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>This is your final opportunity to enter the draw for {work_email}, {collect_phrase} by {artist}.</t>
+          <t>Three days left to collect</t>
         </is>
       </c>
       <c r="C67" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B67,"{artist}",Inputs!$B$4),"{work_email}",Inputs!$B$36),"{collect_phrase}",Inputs!$B$56)</f>
+        <f>B67</f>
         <v/>
       </c>
     </row>
     <row r="68" ht="32" customHeight="1">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>email · last chance, draw · 2</t>
+          <t>email · 3 days · 1</t>
         </is>
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>For a chance to collect, click the link below to enter the draw. The draw closes at {close_time} on {close_weekday}, {close_date_dd}.</t>
+          <t>There are just three days left to collect {collect_phrase} by {artist}.</t>
         </is>
       </c>
       <c r="C68" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B68,"{close_time}",Inputs!$B$53),"{close_weekday}",Inputs!$B$54),"{close_date_dd}",Inputs!$B$55)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="3" t="inlineStr">
-        <is>
-          <t>EMAILS · surveys (LE)</t>
-        </is>
+        <f>SUBSTITUTE(SUBSTITUTE(B68,"{artist}",Inputs!$B$4),"{collect_phrase}",Inputs!$B$59)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69" ht="32" customHeight="1">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>email · 3 days · 2</t>
+        </is>
+      </c>
+      <c r="B69" s="8" t="inlineStr">
+        <is>
+          <t>Click the link to collect before {close_time} on {close_weekday}, {close_date_dd}.</t>
+        </is>
+      </c>
+      <c r="C69" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B69,"{close_time}",Inputs!$B$56),"{close_weekday}",Inputs!$B$57),"{close_date_dd}",Inputs!$B$58)</f>
+        <v/>
       </c>
     </row>
     <row r="70" ht="16" customHeight="1">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>email · first-time survey · subject</t>
+          <t>email · 3 days · footer</t>
         </is>
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>Congratulations on your first Avant Arte edition</t>
+          <t>Add a print to your collection</t>
         </is>
       </c>
       <c r="C70" s="10">
@@ -2352,111 +2403,93 @@
         <v/>
       </c>
     </row>
-    <row r="71" ht="32" customHeight="1">
-      <c r="A71" s="4" t="inlineStr">
-        <is>
-          <t>email · first-time survey · 1</t>
-        </is>
-      </c>
-      <c r="B71" s="8" t="inlineStr">
-        <is>
-          <t>Thank you for adding our collaboration with {artist} to your collection. Great choice!</t>
-        </is>
-      </c>
-      <c r="C71" s="10">
-        <f>SUBSTITUTE(B71,"{artist}",Inputs!$B$4)</f>
-        <v/>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>EMAILS · last chance</t>
+        </is>
       </c>
     </row>
     <row r="72" ht="48" customHeight="1">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>email · first-time survey · 2</t>
+          <t>email · last chance, timed · 1</t>
         </is>
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>I'm {advisor}, an art advisor at Avant Arte. I'm here to connect collectors with artists by making suggestions, answering questions and offering early access to our collaborations.</t>
+          <t>It's now or never for our {ordinal} collaboration with {artist} – {collect_phrase} will be available to order until {close_time} on {close_weekday}, {close_date_dd}.</t>
         </is>
       </c>
       <c r="C72" s="10">
-        <f>SUBSTITUTE(B72,"{advisor}",Inputs!$B$18)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B72,"{artist}",Inputs!$B$4),"{collect_phrase}",Inputs!$B$59),"{ordinal}",Inputs!$B$9),"{close_time}",Inputs!$B$56),"{close_weekday}",Inputs!$B$57),"{close_date_dd}",Inputs!$B$58)</f>
         <v/>
       </c>
     </row>
     <row r="73" ht="32" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>email · first-time survey · 3</t>
+          <t>email · last chance, timed · 2</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>If you have two minutes to complete a short survey about your collecting journey to date, your responses will help guide my recommendations.</t>
+          <t>After this time, the edition size{each_artwork} will be confirmed, and the {work_word} will no longer be available to purchase.</t>
         </is>
       </c>
       <c r="C73" s="10">
-        <f>B73</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74" ht="16" customHeight="1">
+        <f>SUBSTITUTE(SUBSTITUTE(B73,"{each_artwork}",Inputs!$B$65),"{work_word}",Inputs!$B$66)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="32" customHeight="1">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>email · first-time survey · 4</t>
+          <t>email · last chance, draw · 1</t>
         </is>
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>Any questions? Reply to this email.</t>
+          <t>This is your final opportunity to enter the draw for {work_email}, {collect_phrase} by {artist}.</t>
         </is>
       </c>
       <c r="C74" s="10">
-        <f>B74</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75" ht="48" customHeight="1">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B74,"{artist}",Inputs!$B$4),"{work_email}",Inputs!$B$39),"{collect_phrase}",Inputs!$B$59)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75" ht="32" customHeight="1">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>email · non-purchaser survey · 1</t>
+          <t>email · last chance, draw · 2</t>
         </is>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>As someone who registered for updates but ultimately decided not to enter the draw for our collaboration with {artist}, we'd love your feedback.</t>
+          <t>For a chance to collect, click the link below to enter the draw. The draw closes at {close_time} on {close_weekday}, {close_date_dd}.</t>
         </is>
       </c>
       <c r="C75" s="10">
-        <f>SUBSTITUTE(B75,"{artist}",Inputs!$B$4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76" ht="32" customHeight="1">
-      <c r="A76" s="4" t="inlineStr">
-        <is>
-          <t>email · non-purchaser survey · 2</t>
-        </is>
-      </c>
-      <c r="B76" s="8" t="inlineStr">
-        <is>
-          <t>This two-minute survey will guide our future collaborations and help us recommend the right artists and editions for your collection.</t>
-        </is>
-      </c>
-      <c r="C76" s="10">
-        <f>B76</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77" ht="48" customHeight="1">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B75,"{close_time}",Inputs!$B$56),"{close_weekday}",Inputs!$B$57),"{close_date_dd}",Inputs!$B$58)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>EMAILS · surveys (LE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="16" customHeight="1">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>email · non-purchaser survey · 3</t>
+          <t>email · first-time survey · subject</t>
         </is>
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>As a thank you for taking part in the survey and helping us improve the collector experience, you'll be entered into a draw to win a €500 Avant Arte gift card.</t>
+          <t>Congratulations on your first Avant Arte edition</t>
         </is>
       </c>
       <c r="C77" s="10">
@@ -2464,90 +2497,202 @@
         <v/>
       </c>
     </row>
-    <row r="78" ht="16" customHeight="1">
+    <row r="78" ht="32" customHeight="1">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>email · non-purchaser survey · terms</t>
+          <t>email · first-time survey · 1</t>
         </is>
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>You can read the terms here.</t>
+          <t>Thank you for adding our collaboration with {artist} to your collection. Great choice!</t>
         </is>
       </c>
       <c r="C78" s="10">
-        <f>B78</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79" ht="16" customHeight="1">
+        <f>SUBSTITUTE(B78,"{artist}",Inputs!$B$4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79" ht="48" customHeight="1">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>email · non-purchaser survey · footer</t>
+          <t>email · first-time survey · 2</t>
         </is>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>What can we do better?</t>
+          <t>I'm {advisor}, an art advisor at Avant Arte. I'm here to connect collectors with artists by making suggestions, answering questions and offering early access to our collaborations.</t>
         </is>
       </c>
       <c r="C79" s="10">
-        <f>B79</f>
-        <v/>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="3" t="inlineStr">
-        <is>
-          <t>EMAILS · monthly preview</t>
-        </is>
+        <f>SUBSTITUTE(B79,"{advisor}",Inputs!$B$20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80" ht="32" customHeight="1">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>email · first-time survey · 3</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>If you have two minutes to complete a short survey about your collecting journey to date, your responses will help guide my recommendations.</t>
+        </is>
+      </c>
+      <c r="C80" s="10">
+        <f>B80</f>
+        <v/>
       </c>
     </row>
     <row r="81" ht="16" customHeight="1">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>email · monthly preview · opener</t>
+          <t>email · first-time survey · 4</t>
         </is>
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>From {artist} comes {work_intro}{support}.</t>
+          <t>Any questions? Reply to this email.</t>
         </is>
       </c>
       <c r="C81" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B81,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$38),"{support}",Inputs!$B$39)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82" ht="32" customHeight="1">
+        <f>B81</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82" ht="48" customHeight="1">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>email · monthly preview · when, draw</t>
+          <t>email · non-purchaser survey · 1</t>
         </is>
       </c>
       <c r="B82" s="8" t="inlineStr">
         <is>
-          <t>The edition will be allocated by a randomised draw, which closes at {close_time} on {close_date}.</t>
+          <t>As someone who registered for updates but ultimately decided not to enter the draw for our collaboration with {artist}, we'd love your feedback.</t>
         </is>
       </c>
       <c r="C82" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B82,"{close_date}",Inputs!$B$52),"{close_time}",Inputs!$B$53)</f>
+        <f>SUBSTITUTE(B82,"{artist}",Inputs!$B$4)</f>
         <v/>
       </c>
     </row>
     <row r="83" ht="32" customHeight="1">
       <c r="A83" s="4" t="inlineStr">
         <is>
+          <t>email · non-purchaser survey · 2</t>
+        </is>
+      </c>
+      <c r="B83" s="8" t="inlineStr">
+        <is>
+          <t>This two-minute survey will guide our future collaborations and help us recommend the right artists and editions for your collection.</t>
+        </is>
+      </c>
+      <c r="C83" s="10">
+        <f>B83</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84" ht="48" customHeight="1">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>email · non-purchaser survey · 3</t>
+        </is>
+      </c>
+      <c r="B84" s="8" t="inlineStr">
+        <is>
+          <t>As a thank you for taking part in the survey and helping us improve the collector experience, you'll be entered into a draw to win a €500 Avant Arte gift card.</t>
+        </is>
+      </c>
+      <c r="C84" s="10">
+        <f>B84</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85" ht="16" customHeight="1">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>email · non-purchaser survey · terms</t>
+        </is>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>You can read the terms here.</t>
+        </is>
+      </c>
+      <c r="C85" s="10">
+        <f>B85</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86" ht="16" customHeight="1">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>email · non-purchaser survey · footer</t>
+        </is>
+      </c>
+      <c r="B86" s="8" t="inlineStr">
+        <is>
+          <t>What can we do better?</t>
+        </is>
+      </c>
+      <c r="C86" s="10">
+        <f>B86</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>EMAILS · monthly preview</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="16" customHeight="1">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>email · monthly preview · opener</t>
+        </is>
+      </c>
+      <c r="B88" s="8" t="inlineStr">
+        <is>
+          <t>From {artist} comes {work_intro}{support}.</t>
+        </is>
+      </c>
+      <c r="C88" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B88,"{artist}",Inputs!$B$4),"{work_intro}",Inputs!$B$41),"{support}",Inputs!$B$42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89" ht="32" customHeight="1">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>email · monthly preview · when, draw</t>
+        </is>
+      </c>
+      <c r="B89" s="8" t="inlineStr">
+        <is>
+          <t>The edition will be allocated by a randomised draw, which closes at {close_time} on {close_date}.</t>
+        </is>
+      </c>
+      <c r="C89" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(B89,"{close_date}",Inputs!$B$55),"{close_time}",Inputs!$B$56)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90" ht="32" customHeight="1">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
           <t>email · monthly preview · when, timed</t>
         </is>
       </c>
-      <c r="B83" s="8" t="inlineStr">
+      <c r="B90" s="8" t="inlineStr">
         <is>
           <t>The edition will be available to collect for {window} only, from {launch_time} on {launch_weekday}, {launch_date_dd}.</t>
         </is>
       </c>
-      <c r="C83" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B83,"{window}",Inputs!$B$13),"{launch_time}",Inputs!$B$49),"{launch_weekday}",Inputs!$B$50),"{launch_date_dd}",Inputs!$B$51)</f>
+      <c r="C90" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B90,"{window}",Inputs!$B$15),"{launch_time}",Inputs!$B$52),"{launch_weekday}",Inputs!$B$53),"{launch_date_dd}",Inputs!$B$54)</f>
         <v/>
       </c>
     </row>
@@ -2562,19 +2707,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="56" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="56" customWidth="1" min="6" max="6"/>
     <col width="44" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="92" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="92" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2587,7 +2733,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Every cell below is a formula over Inputs and Lines. Skeleton: status line · substance · features line · action line · hashtag. Coming Soon opens with the bio.</t>
+          <t>Every cell below is a formula over Inputs and Lines. Skeleton: status line · substance · features line · action line · hashtag. Coming Soon opens with the bio. The Insiders account posts the same caption; Channels says which.</t>
         </is>
       </c>
     </row>
@@ -2604,40 +2750,45 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
+          <t>Channels</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
           <t>Made of</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Status line</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Substance</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Features line</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Action line</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Hashtag</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Caption</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>Characters</t>
         </is>
@@ -2654,35 +2805,40 @@
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
           <t>bio · status · action</t>
         </is>
       </c>
-      <c r="D4" s="11">
+      <c r="E4" s="11">
         <f>Lines!$C$5</f>
         <v/>
       </c>
-      <c r="E4" s="11">
-        <f>Inputs!$B$41</f>
-        <v/>
-      </c>
       <c r="F4" s="11">
-        <f>""</f>
+        <f>Inputs!$B$44</f>
         <v/>
       </c>
       <c r="G4" s="11">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="H4" s="11">
         <f>Lines!$C$21</f>
         <v/>
       </c>
-      <c r="H4" s="11">
-        <f>""</f>
-        <v/>
-      </c>
       <c r="I4" s="11">
-        <f>E4&amp;IF(D4="","",CHAR(10)&amp;CHAR(10)&amp;D4)&amp;IF(G4="","",CHAR(10)&amp;CHAR(10)&amp;G4)</f>
+        <f>""</f>
         <v/>
       </c>
       <c r="J4" s="11">
-        <f>LEN(I4)</f>
+        <f>F4&amp;IF(E4="","",CHAR(10)&amp;CHAR(10)&amp;E4)&amp;IF(H4="","",CHAR(10)&amp;CHAR(10)&amp;H4)</f>
+        <v/>
+      </c>
+      <c r="K4" s="11">
+        <f>LEN(J4)</f>
         <v/>
       </c>
     </row>
@@ -2697,35 +2853,40 @@
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
+          <t>Main + Insiders</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
           <t>status · hook · features + beneficiary · action · hashtag</t>
         </is>
       </c>
-      <c r="D5" s="11">
-        <f>IF(Inputs!$B$9="yes",Lines!$C$7,Lines!$C$6)</f>
-        <v/>
-      </c>
       <c r="E5" s="11">
-        <f>Inputs!$B$28</f>
+        <f>IF(Inputs!$B$11="yes",Lines!$C$7,Lines!$C$6)</f>
         <v/>
       </c>
       <c r="F5" s="11">
-        <f>Lines!$C$15&amp;IF(Inputs!$B$42,"",IF(Inputs!$B$40="",""," "&amp;Lines!$C$16))</f>
+        <f>Inputs!$B$30</f>
         <v/>
       </c>
       <c r="G5" s="11">
-        <f>IF(Inputs!$B$12="draw",Lines!$C$18,Lines!$C$17)</f>
+        <f>Lines!$C$15&amp;IF(Inputs!$B$45,"",IF(Inputs!$B$43="",""," "&amp;Lines!$C$16))</f>
         <v/>
       </c>
       <c r="H5" s="11">
-        <f>IF(Inputs!$B$6="","",Lines!$C$22)</f>
+        <f>IF(Inputs!$B$14="draw",Lines!$C$18,Lines!$C$17)</f>
         <v/>
       </c>
       <c r="I5" s="11">
-        <f>D5&amp;IF(E5="","",CHAR(10)&amp;CHAR(10)&amp;E5)&amp;IF(F5="","",CHAR(10)&amp;CHAR(10)&amp;F5)&amp;IF(G5="","",CHAR(10)&amp;CHAR(10)&amp;G5)&amp;IF(H5="","",CHAR(10)&amp;CHAR(10)&amp;H5)</f>
+        <f>IF(Inputs!$B$8="","",Lines!$C$22)</f>
         <v/>
       </c>
       <c r="J5" s="11">
-        <f>LEN(I5)</f>
+        <f>E5&amp;IF(F5="","",CHAR(10)&amp;CHAR(10)&amp;F5)&amp;IF(G5="","",CHAR(10)&amp;CHAR(10)&amp;G5)&amp;IF(H5="","",CHAR(10)&amp;CHAR(10)&amp;H5)&amp;IF(I5="","",CHAR(10)&amp;CHAR(10)&amp;I5)</f>
+        <v/>
+      </c>
+      <c r="K5" s="11">
+        <f>LEN(J5)</f>
         <v/>
       </c>
     </row>
@@ -2740,35 +2901,40 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
           <t>status · making · features + beneficiary · action</t>
         </is>
       </c>
-      <c r="D6" s="11">
+      <c r="E6" s="11">
         <f>Lines!$C$8</f>
         <v/>
       </c>
-      <c r="E6" s="11">
-        <f>Inputs!$B$47</f>
-        <v/>
-      </c>
       <c r="F6" s="11">
-        <f>Lines!$C$15&amp;IF(Inputs!$B$40="",""," "&amp;Lines!$C$16)</f>
+        <f>Inputs!$B$50</f>
         <v/>
       </c>
       <c r="G6" s="11">
-        <f>IF(Inputs!$B$12="draw",Lines!$C$18,Lines!$C$17)</f>
+        <f>Lines!$C$15&amp;IF(Inputs!$B$43="",""," "&amp;Lines!$C$16)</f>
         <v/>
       </c>
       <c r="H6" s="11">
-        <f>""</f>
+        <f>IF(Inputs!$B$14="draw",Lines!$C$18,Lines!$C$17)</f>
         <v/>
       </c>
       <c r="I6" s="11">
-        <f>D6&amp;IF(E6="","",CHAR(10)&amp;CHAR(10)&amp;E6)&amp;IF(F6="","",CHAR(10)&amp;CHAR(10)&amp;F6)&amp;IF(G6="","",CHAR(10)&amp;CHAR(10)&amp;G6)</f>
+        <f>""</f>
         <v/>
       </c>
       <c r="J6" s="11">
-        <f>LEN(I6)</f>
+        <f>E6&amp;IF(F6="","",CHAR(10)&amp;CHAR(10)&amp;F6)&amp;IF(G6="","",CHAR(10)&amp;CHAR(10)&amp;G6)&amp;IF(H6="","",CHAR(10)&amp;CHAR(10)&amp;H6)</f>
+        <v/>
+      </c>
+      <c r="K6" s="11">
+        <f>LEN(J6)</f>
         <v/>
       </c>
     </row>
@@ -2783,35 +2949,40 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
           <t>quote · status · features + beneficiary · action</t>
         </is>
       </c>
-      <c r="D7" s="11">
-        <f>IF(Inputs!$B$30="","(no quote given, post skipped)",Lines!$C$9)</f>
-        <v/>
-      </c>
       <c r="E7" s="11">
-        <f>IF(Inputs!$B$30="","",Lines!$C$10)</f>
+        <f>IF(Inputs!$B$32="","(no quote given, post skipped)",Lines!$C$9)</f>
         <v/>
       </c>
       <c r="F7" s="11">
-        <f>IF(Inputs!$B$30="","",Lines!$C$15&amp;IF(Inputs!$B$40="",""," "&amp;Lines!$C$16))</f>
+        <f>IF(Inputs!$B$32="","",Lines!$C$10)</f>
         <v/>
       </c>
       <c r="G7" s="11">
-        <f>IF(Inputs!$B$30="","",IF(Inputs!$B$12="draw",Lines!$C$18,Lines!$C$17))</f>
+        <f>IF(Inputs!$B$32="","",Lines!$C$15&amp;IF(Inputs!$B$43="",""," "&amp;Lines!$C$16))</f>
         <v/>
       </c>
       <c r="H7" s="11">
-        <f>""</f>
+        <f>IF(Inputs!$B$32="","",IF(Inputs!$B$14="draw",Lines!$C$18,Lines!$C$17))</f>
         <v/>
       </c>
       <c r="I7" s="11">
-        <f>IF(Inputs!$B$30="","(no quote given, post skipped)",D7&amp;IF(E7="","",CHAR(10)&amp;CHAR(10)&amp;E7)&amp;IF(F7="","",CHAR(10)&amp;CHAR(10)&amp;F7)&amp;IF(G7="","",CHAR(10)&amp;CHAR(10)&amp;G7))</f>
+        <f>""</f>
         <v/>
       </c>
       <c r="J7" s="11">
-        <f>LEN(I7)</f>
+        <f>IF(Inputs!$B$32="","(no quote given, post skipped)",E7&amp;IF(F7="","",CHAR(10)&amp;CHAR(10)&amp;F7)&amp;IF(G7="","",CHAR(10)&amp;CHAR(10)&amp;G7)&amp;IF(H7="","",CHAR(10)&amp;CHAR(10)&amp;H7))</f>
+        <v/>
+      </c>
+      <c r="K7" s="11">
+        <f>LEN(J7)</f>
         <v/>
       </c>
     </row>
@@ -2826,35 +2997,40 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
+          <t>Main + Insiders</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
           <t>status · features + beneficiary · action</t>
         </is>
       </c>
-      <c r="D8" s="11">
-        <f>IF(Inputs!$B$12="draw","(not used for a draw)",Lines!$C$11)</f>
-        <v/>
-      </c>
       <c r="E8" s="11">
-        <f>""</f>
+        <f>IF(Inputs!$B$14="draw","(not used for a draw)",Lines!$C$11)</f>
         <v/>
       </c>
       <c r="F8" s="11">
-        <f>IF(Inputs!$B$12="draw","",Lines!$C$15&amp;IF(Inputs!$B$40="",""," "&amp;Lines!$C$16))</f>
+        <f>""</f>
         <v/>
       </c>
       <c r="G8" s="11">
-        <f>IF(Inputs!$B$12="draw","",IF(Inputs!$B$12="draw",Lines!$C$20,Lines!$C$19))</f>
+        <f>IF(Inputs!$B$14="draw","",Lines!$C$15&amp;IF(Inputs!$B$43="",""," "&amp;Lines!$C$16))</f>
         <v/>
       </c>
       <c r="H8" s="11">
-        <f>""</f>
+        <f>IF(Inputs!$B$14="draw","",IF(Inputs!$B$14="draw",Lines!$C$20,Lines!$C$19))</f>
         <v/>
       </c>
       <c r="I8" s="11">
-        <f>IF(Inputs!$B$12="draw","(not used for a draw)",D8&amp;IF(F8="","",CHAR(10)&amp;CHAR(10)&amp;F8)&amp;IF(G8="","",CHAR(10)&amp;CHAR(10)&amp;G8))</f>
+        <f>""</f>
         <v/>
       </c>
       <c r="J8" s="11">
-        <f>LEN(I8)</f>
+        <f>IF(Inputs!$B$14="draw","(not used for a draw)",E8&amp;IF(G8="","",CHAR(10)&amp;CHAR(10)&amp;G8)&amp;IF(H8="","",CHAR(10)&amp;CHAR(10)&amp;H8))</f>
+        <v/>
+      </c>
+      <c r="K8" s="11">
+        <f>LEN(J8)</f>
         <v/>
       </c>
     </row>
@@ -2869,35 +3045,40 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
+          <t>Main + Insiders (the plan's Halfway through)</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
           <t>status · features + beneficiary · action</t>
         </is>
       </c>
-      <c r="D9" s="11">
-        <f>IF(Inputs!$B$12="draw","(not used for a draw)",Lines!$C$12)</f>
-        <v/>
-      </c>
       <c r="E9" s="11">
-        <f>""</f>
+        <f>IF(Inputs!$B$14="draw","(not used for a draw)",Lines!$C$12)</f>
         <v/>
       </c>
       <c r="F9" s="11">
-        <f>IF(Inputs!$B$12="draw","",Lines!$C$15&amp;IF(Inputs!$B$40="",""," "&amp;Lines!$C$16))</f>
+        <f>""</f>
         <v/>
       </c>
       <c r="G9" s="11">
-        <f>IF(Inputs!$B$12="draw","",IF(Inputs!$B$12="draw",Lines!$C$20,Lines!$C$19))</f>
+        <f>IF(Inputs!$B$14="draw","",Lines!$C$15&amp;IF(Inputs!$B$43="",""," "&amp;Lines!$C$16))</f>
         <v/>
       </c>
       <c r="H9" s="11">
-        <f>""</f>
+        <f>IF(Inputs!$B$14="draw","",IF(Inputs!$B$14="draw",Lines!$C$20,Lines!$C$19))</f>
         <v/>
       </c>
       <c r="I9" s="11">
-        <f>IF(Inputs!$B$12="draw","(not used for a draw)",D9&amp;IF(F9="","",CHAR(10)&amp;CHAR(10)&amp;F9)&amp;IF(G9="","",CHAR(10)&amp;CHAR(10)&amp;G9))</f>
+        <f>""</f>
         <v/>
       </c>
       <c r="J9" s="11">
-        <f>LEN(I9)</f>
+        <f>IF(Inputs!$B$14="draw","(not used for a draw)",E9&amp;IF(G9="","",CHAR(10)&amp;CHAR(10)&amp;G9)&amp;IF(H9="","",CHAR(10)&amp;CHAR(10)&amp;H9))</f>
+        <v/>
+      </c>
+      <c r="K9" s="11">
+        <f>LEN(J9)</f>
         <v/>
       </c>
     </row>
@@ -2912,35 +3093,40 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
           <t>status · features + beneficiary · action</t>
         </is>
       </c>
-      <c r="D10" s="11">
-        <f>IF(Inputs!$B$12="draw",Lines!$C$14,Lines!$C$13)</f>
-        <v/>
-      </c>
       <c r="E10" s="11">
-        <f>""</f>
+        <f>IF(Inputs!$B$14="draw",Lines!$C$14,Lines!$C$13)</f>
         <v/>
       </c>
       <c r="F10" s="11">
-        <f>Lines!$C$15&amp;IF(Inputs!$B$40="",""," "&amp;Lines!$C$16)</f>
+        <f>""</f>
         <v/>
       </c>
       <c r="G10" s="11">
-        <f>IF(Inputs!$B$12="draw",Lines!$C$20,Lines!$C$19)</f>
+        <f>Lines!$C$15&amp;IF(Inputs!$B$43="",""," "&amp;Lines!$C$16)</f>
         <v/>
       </c>
       <c r="H10" s="11">
-        <f>""</f>
+        <f>IF(Inputs!$B$14="draw",Lines!$C$20,Lines!$C$19)</f>
         <v/>
       </c>
       <c r="I10" s="11">
-        <f>D10&amp;IF(F10="","",CHAR(10)&amp;CHAR(10)&amp;F10)&amp;IF(G10="","",CHAR(10)&amp;CHAR(10)&amp;G10)</f>
+        <f>""</f>
         <v/>
       </c>
       <c r="J10" s="11">
-        <f>LEN(I10)</f>
+        <f>E10&amp;IF(G10="","",CHAR(10)&amp;CHAR(10)&amp;G10)&amp;IF(H10="","",CHAR(10)&amp;CHAR(10)&amp;H10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="11">
+        <f>LEN(J10)</f>
         <v/>
       </c>
     </row>
@@ -2950,6 +3136,287 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="80" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>The tweets, assembled</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>The post's status line with the X handle, the hook on the announcement only, the beneficiary named once, and an action line that ends with the link. No features line, no hashtag, no bio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Tweet</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Made of</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Status line</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Substance</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Beneficiary line</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Action line</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Tweet</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Characters</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>coming soon</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>status · action</t>
+        </is>
+      </c>
+      <c r="D4" s="11">
+        <f>Lines!$C$24</f>
+        <v/>
+      </c>
+      <c r="E4" s="11">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="F4" s="11">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="G4" s="11">
+        <f>Lines!$C$25</f>
+        <v/>
+      </c>
+      <c r="H4" s="11">
+        <f>D4&amp;IF(G4="","",CHAR(10)&amp;CHAR(10)&amp;G4)</f>
+        <v/>
+      </c>
+      <c r="I4" s="11">
+        <f>LEN(H4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="150" customHeight="1">
+      <c r="A5" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>announce</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>status · hook · beneficiary · action</t>
+        </is>
+      </c>
+      <c r="D5" s="11">
+        <f>SUBSTITUTE(IF(Inputs!$B$11="yes",Lines!$C$7,Lines!$C$6),Inputs!$B$35,Inputs!$B$36)</f>
+        <v/>
+      </c>
+      <c r="E5" s="11">
+        <f>Inputs!$B$30</f>
+        <v/>
+      </c>
+      <c r="F5" s="11">
+        <f>IF(OR(Inputs!$B$18="",Inputs!$B$45),"",Lines!$C$26)</f>
+        <v/>
+      </c>
+      <c r="G5" s="11">
+        <f>IF(Inputs!$B$14="draw",Lines!$C$28,Lines!$C$27)</f>
+        <v/>
+      </c>
+      <c r="H5" s="11">
+        <f>D5&amp;IF(E5="","",CHAR(10)&amp;CHAR(10)&amp;E5)&amp;IF(F5="","",CHAR(10)&amp;CHAR(10)&amp;F5)&amp;IF(G5="","",CHAR(10)&amp;CHAR(10)&amp;G5)</f>
+        <v/>
+      </c>
+      <c r="I5" s="11">
+        <f>LEN(H5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>live (timed only)</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>status · action</t>
+        </is>
+      </c>
+      <c r="D6" s="11">
+        <f>IF(Inputs!$B$14="draw","(not used for a draw)",SUBSTITUTE(Lines!$C$11,Inputs!$B$35,Inputs!$B$36))</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
+        <f>IF(Inputs!$B$14="draw","",IF(Inputs!$B$14="draw",Lines!$C$28,Lines!$C$29))</f>
+        <v/>
+      </c>
+      <c r="H6" s="11">
+        <f>IF(Inputs!$B$14="draw","(not used for a draw)",D6&amp;IF(G6="","",CHAR(10)&amp;CHAR(10)&amp;G6))</f>
+        <v/>
+      </c>
+      <c r="I6" s="11">
+        <f>LEN(H6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>still time (timed only)</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>status · action</t>
+        </is>
+      </c>
+      <c r="D7" s="11">
+        <f>IF(Inputs!$B$14="draw","(not used for a draw)",SUBSTITUTE(Lines!$C$12,Inputs!$B$35,Inputs!$B$36))</f>
+        <v/>
+      </c>
+      <c r="E7" s="11">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="F7" s="11">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="G7" s="11">
+        <f>IF(Inputs!$B$14="draw","",IF(Inputs!$B$14="draw",Lines!$C$28,Lines!$C$29))</f>
+        <v/>
+      </c>
+      <c r="H7" s="11">
+        <f>IF(Inputs!$B$14="draw","(not used for a draw)",D7&amp;IF(G7="","",CHAR(10)&amp;CHAR(10)&amp;G7))</f>
+        <v/>
+      </c>
+      <c r="I7" s="11">
+        <f>LEN(H7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="80" customHeight="1">
+      <c r="A8" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>last chance</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>status · action</t>
+        </is>
+      </c>
+      <c r="D8" s="11">
+        <f>IF(Inputs!$B$14="draw",SUBSTITUTE(Lines!$C$14,Inputs!$B$35,Inputs!$B$36),SUBSTITUTE(Lines!$C$13,Inputs!$B$35,Inputs!$B$36))</f>
+        <v/>
+      </c>
+      <c r="E8" s="11">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="F8" s="11">
+        <f>""</f>
+        <v/>
+      </c>
+      <c r="G8" s="11">
+        <f>IF(Inputs!$B$14="draw",Lines!$C$28,Lines!$C$29)</f>
+        <v/>
+      </c>
+      <c r="H8" s="11">
+        <f>D8&amp;IF(G8="","",CHAR(10)&amp;CHAR(10)&amp;G8)</f>
+        <v/>
+      </c>
+      <c r="I8" s="11">
+        <f>LEN(H8)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3085,39 +3552,39 @@
         <v/>
       </c>
       <c r="E4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",Lines!$C$29)</f>
+        <f>IF($D4&lt;&gt;"yes","",Lines!$C$36)</f>
         <v/>
       </c>
       <c r="F4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$12="draw","Enter the draw for a chance to collect. Closes "&amp;Inputs!$B$52&amp;".","Launching "&amp;Inputs!$B$48&amp;". Register for updates."))</f>
+        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$14="draw","Enter the draw for a chance to collect. Closes "&amp;Inputs!$B$55&amp;".","Launching "&amp;Inputs!$B$51&amp;". Register for updates."))</f>
         <v/>
       </c>
       <c r="G4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$12="draw","Enter the draw","Launching "&amp;Inputs!$B$48))</f>
+        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$14="draw","Enter the draw","Launching "&amp;Inputs!$B$51))</f>
         <v/>
       </c>
       <c r="H4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$12="draw",Inputs!$B$37,Inputs!$B$37&amp;" by "&amp;Inputs!$B$4))</f>
+        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$14="draw",Inputs!$B$40,Inputs!$B$40&amp;" by "&amp;Inputs!$B$4))</f>
         <v/>
       </c>
       <c r="I4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",(Lines!$C$30&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$46&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$44&amp;CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$12="draw",Lines!$C$26,(Lines!$C$31&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$32))))</f>
+        <f>IF($D4&lt;&gt;"yes","",(Lines!$C$37&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$30&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$49&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$47&amp;CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$14="draw",Lines!$C$33,(Lines!$C$38&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$39))))</f>
         <v/>
       </c>
       <c r="J4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$12="draw","Enter the draw","Discover the collaboration"))</f>
+        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$14="draw","Enter the draw","Discover the collaboration"))</f>
         <v/>
       </c>
       <c r="K4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",Inputs!$B$60)</f>
+        <f>IF($D4&lt;&gt;"yes","",Inputs!$B$63)</f>
         <v/>
       </c>
       <c r="L4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",Inputs!$B$61)</f>
+        <f>IF($D4&lt;&gt;"yes","",Inputs!$B$64)</f>
         <v/>
       </c>
       <c r="M4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$12="draw","Collect "&amp;Inputs!$B$56,"Launching "&amp;Inputs!$B$48))</f>
+        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$14="draw","Collect "&amp;Inputs!$B$59,"Launching "&amp;Inputs!$B$51))</f>
         <v/>
       </c>
       <c r="N4" s="11">
@@ -3144,7 +3611,7 @@
         </is>
       </c>
       <c r="D5" s="11">
-        <f>IF(Inputs!$B$12="draw","(not used for a draw)","yes")</f>
+        <f>IF(Inputs!$B$14="draw","(not used for a draw)","yes")</f>
         <v/>
       </c>
       <c r="E5" s="11">
@@ -3164,7 +3631,7 @@
         <v/>
       </c>
       <c r="I5" s="11">
-        <f>IF($D5&lt;&gt;"yes","",(Lines!$C$34&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$35&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$36&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$37))</f>
+        <f>IF($D5&lt;&gt;"yes","",(Lines!$C$41&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$42&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$43&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$44))</f>
         <v/>
       </c>
       <c r="J5" s="11">
@@ -3207,7 +3674,7 @@
         </is>
       </c>
       <c r="D6" s="11">
-        <f>IF(Inputs!$B$12="draw","(not used for a draw)","yes")</f>
+        <f>IF(Inputs!$B$14="draw","(not used for a draw)","yes")</f>
         <v/>
       </c>
       <c r="E6" s="11">
@@ -3227,7 +3694,7 @@
         <v/>
       </c>
       <c r="I6" s="11">
-        <f>IF($D6&lt;&gt;"yes","",(Lines!$C$24&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$39&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$45&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$40&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$42))</f>
+        <f>IF($D6&lt;&gt;"yes","",(Lines!$C$31&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$46&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$30&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$48&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$47&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$49))</f>
         <v/>
       </c>
       <c r="J6" s="11">
@@ -3270,7 +3737,7 @@
         </is>
       </c>
       <c r="D7" s="11">
-        <f>IF(Inputs!$B$12="draw","(not used for a draw)","yes")</f>
+        <f>IF(Inputs!$B$14="draw","(not used for a draw)","yes")</f>
         <v/>
       </c>
       <c r="E7" s="11">
@@ -3290,7 +3757,7 @@
         <v/>
       </c>
       <c r="I7" s="11">
-        <f>IF($D7&lt;&gt;"yes","",(Lines!$C$24&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$39&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$45&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$41&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$42&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$27&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$25))</f>
+        <f>IF($D7&lt;&gt;"yes","",(Lines!$C$31&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$46&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$30&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$48&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$48&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$49&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$34&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$32))</f>
         <v/>
       </c>
       <c r="J7" s="11">
@@ -3298,7 +3765,7 @@
         <v/>
       </c>
       <c r="K7" s="11">
-        <f>IF($D7&lt;&gt;"yes","",Inputs!$B$60)</f>
+        <f>IF($D7&lt;&gt;"yes","",Inputs!$B$63)</f>
         <v/>
       </c>
       <c r="L7" s="11">
@@ -3341,7 +3808,7 @@
         <v/>
       </c>
       <c r="F8" s="11">
-        <f>IF($D8&lt;&gt;"yes","",IF(Inputs!$B$12="draw","A first look, plus early access to a limited number of pre-orders.","Collect 24 hours before everyone else."))</f>
+        <f>IF($D8&lt;&gt;"yes","",IF(Inputs!$B$14="draw","A first look, plus early access to a limited number of pre-orders.","Collect 24 hours before everyone else."))</f>
         <v/>
       </c>
       <c r="G8" s="11">
@@ -3353,7 +3820,7 @@
         <v/>
       </c>
       <c r="I8" s="11">
-        <f>IF($D8&lt;&gt;"yes","",(Lines!$C$24&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$46&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$12="draw",Lines!$C$47,Lines!$C$48)&amp;CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$12="draw",Lines!$C$49,Lines!$C$50)&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$25&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$51))</f>
+        <f>IF($D8&lt;&gt;"yes","",(Lines!$C$31&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$53&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$30&amp;CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$14="draw",Lines!$C$54,Lines!$C$55)&amp;CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$14="draw",Lines!$C$56,Lines!$C$57)&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$32&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$58))</f>
         <v/>
       </c>
       <c r="J8" s="11">
@@ -3361,7 +3828,7 @@
         <v/>
       </c>
       <c r="K8" s="11">
-        <f>IF($D8&lt;&gt;"yes","",Inputs!$B$60)</f>
+        <f>IF($D8&lt;&gt;"yes","",Inputs!$B$63)</f>
         <v/>
       </c>
       <c r="L8" s="11">
@@ -3369,7 +3836,7 @@
         <v/>
       </c>
       <c r="M8" s="11">
-        <f>IF($D8&lt;&gt;"yes","",IF(Inputs!$B$12="draw","Especially for you.","24 hours ahead of the public launch"))</f>
+        <f>IF($D8&lt;&gt;"yes","",IF(Inputs!$B$14="draw","Especially for you.","24 hours ahead of the public launch"))</f>
         <v/>
       </c>
       <c r="N8" s="11">
@@ -3396,7 +3863,7 @@
         </is>
       </c>
       <c r="D9" s="11">
-        <f>IF(Inputs!$B$12="draw","yes","(not used for a timed edition)")</f>
+        <f>IF(Inputs!$B$14="draw","yes","(not used for a timed edition)")</f>
         <v/>
       </c>
       <c r="E9" s="11">
@@ -3416,7 +3883,7 @@
         <v/>
       </c>
       <c r="I9" s="11">
-        <f>IF($D9&lt;&gt;"yes","",(Lines!$C$24&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$43&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$44&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$45&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$27&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$25))</f>
+        <f>IF($D9&lt;&gt;"yes","",(Lines!$C$31&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$50&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$30&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$51&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$52&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$34&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$32))</f>
         <v/>
       </c>
       <c r="J9" s="11">
@@ -3424,7 +3891,7 @@
         <v/>
       </c>
       <c r="K9" s="11">
-        <f>IF($D9&lt;&gt;"yes","",Inputs!$B$60)</f>
+        <f>IF($D9&lt;&gt;"yes","",Inputs!$B$63)</f>
         <v/>
       </c>
       <c r="L9" s="11">
@@ -3459,15 +3926,15 @@
         </is>
       </c>
       <c r="D10" s="11">
-        <f>IF(Inputs!$B$12="draw","(not used for a draw)","yes")</f>
+        <f>IF(Inputs!$B$14="draw","(not used for a draw)","yes")</f>
         <v/>
       </c>
       <c r="E10" s="11">
-        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$4&amp;" – Available now, for "&amp;Inputs!$B$13&amp;" only")</f>
+        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$4&amp;" – Available now, for "&amp;Inputs!$B$15&amp;" only")</f>
         <v/>
       </c>
       <c r="F10" s="11">
-        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$58&amp;", starting now.")</f>
+        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$61&amp;", starting now.")</f>
         <v/>
       </c>
       <c r="G10" s="11">
@@ -3475,11 +3942,11 @@
         <v/>
       </c>
       <c r="H10" s="11">
-        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$58&amp;", starting now")</f>
+        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$61&amp;", starting now")</f>
         <v/>
       </c>
       <c r="I10" s="11">
-        <f>IF($D10&lt;&gt;"yes","",(Lines!$C$53&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$46&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$45&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$54))</f>
+        <f>IF($D10&lt;&gt;"yes","",(Lines!$C$60&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$30&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$49&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$48&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$61))</f>
         <v/>
       </c>
       <c r="J10" s="11">
@@ -3487,15 +3954,15 @@
         <v/>
       </c>
       <c r="K10" s="11">
-        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$60)</f>
+        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$63)</f>
         <v/>
       </c>
       <c r="L10" s="11">
-        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$61)</f>
+        <f>IF($D10&lt;&gt;"yes","",Inputs!$B$64)</f>
         <v/>
       </c>
       <c r="M10" s="11">
-        <f>IF($D10&lt;&gt;"yes","","Collect "&amp;Inputs!$B$56)</f>
+        <f>IF($D10&lt;&gt;"yes","","Collect "&amp;Inputs!$B$59)</f>
         <v/>
       </c>
       <c r="N10" s="11">
@@ -3522,7 +3989,7 @@
         </is>
       </c>
       <c r="D11" s="11">
-        <f>IF(Inputs!$B$12="draw","(not used for a draw)",IF(Inputs!$B$13="48 hours","yes","(48-hour windows only; a one-week window gets the 5 days and 3 days emails)"))</f>
+        <f>IF(Inputs!$B$14="draw","(not used for a draw)",IF(Inputs!$B$15="48 hours","yes","(48-hour windows only; a one-week window gets the 5 days and 3 days emails)"))</f>
         <v/>
       </c>
       <c r="E11" s="11">
@@ -3534,11 +4001,11 @@
         <v/>
       </c>
       <c r="G11" s="11">
-        <f>IF($D11&lt;&gt;"yes","",Lines!$C$55)</f>
+        <f>IF($D11&lt;&gt;"yes","",Lines!$C$62)</f>
         <v/>
       </c>
       <c r="H11" s="11">
-        <f>IF($D11&lt;&gt;"yes","",Lines!$C$56)</f>
+        <f>IF($D11&lt;&gt;"yes","",Lines!$C$63)</f>
         <v/>
       </c>
       <c r="I11" s="11">
@@ -3558,7 +4025,7 @@
         <v/>
       </c>
       <c r="M11" s="11">
-        <f>IF($D11&lt;&gt;"yes","",Lines!$C$57)</f>
+        <f>IF($D11&lt;&gt;"yes","",Lines!$C$64)</f>
         <v/>
       </c>
       <c r="N11" s="11">
@@ -3585,7 +4052,7 @@
         </is>
       </c>
       <c r="D12" s="11">
-        <f>IF(Inputs!$B$12="draw","(not used for a draw)",IF(Inputs!$B$13="48 hours","(one-week windows only; a 48-hour window gets the halfway email)","yes"))</f>
+        <f>IF(Inputs!$B$14="draw","(not used for a draw)",IF(Inputs!$B$15="48 hours","(one-week windows only; a 48-hour window gets the halfway email)","yes"))</f>
         <v/>
       </c>
       <c r="E12" s="11">
@@ -3597,11 +4064,11 @@
         <v/>
       </c>
       <c r="G12" s="11">
-        <f>IF($D12&lt;&gt;"yes","",Lines!$C$55)</f>
+        <f>IF($D12&lt;&gt;"yes","",Lines!$C$62)</f>
         <v/>
       </c>
       <c r="H12" s="11">
-        <f>IF($D12&lt;&gt;"yes","",Lines!$C$58)</f>
+        <f>IF($D12&lt;&gt;"yes","",Lines!$C$65)</f>
         <v/>
       </c>
       <c r="I12" s="11">
@@ -3621,7 +4088,7 @@
         <v/>
       </c>
       <c r="M12" s="11">
-        <f>IF($D12&lt;&gt;"yes","",Lines!$C$59)</f>
+        <f>IF($D12&lt;&gt;"yes","",Lines!$C$66)</f>
         <v/>
       </c>
       <c r="N12" s="11">
@@ -3648,7 +4115,7 @@
         </is>
       </c>
       <c r="D13" s="11">
-        <f>IF(Inputs!$B$12="draw","(not used for a draw)",IF(Inputs!$B$13="48 hours","(one-week windows only; a 48-hour window gets the halfway email)","yes"))</f>
+        <f>IF(Inputs!$B$14="draw","(not used for a draw)",IF(Inputs!$B$15="48 hours","(one-week windows only; a 48-hour window gets the halfway email)","yes"))</f>
         <v/>
       </c>
       <c r="E13" s="11">
@@ -3660,15 +4127,15 @@
         <v/>
       </c>
       <c r="G13" s="11">
-        <f>IF($D13&lt;&gt;"yes","",Inputs!$B$37&amp;" by "&amp;Inputs!$B$4)</f>
+        <f>IF($D13&lt;&gt;"yes","",Inputs!$B$40&amp;" by "&amp;Inputs!$B$4)</f>
         <v/>
       </c>
       <c r="H13" s="11">
-        <f>IF($D13&lt;&gt;"yes","",Lines!$C$60)</f>
+        <f>IF($D13&lt;&gt;"yes","",Lines!$C$67)</f>
         <v/>
       </c>
       <c r="I13" s="11">
-        <f>IF($D13&lt;&gt;"yes","",(Lines!$C$61&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$62))</f>
+        <f>IF($D13&lt;&gt;"yes","",(Lines!$C$68&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$30&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$69))</f>
         <v/>
       </c>
       <c r="J13" s="11">
@@ -3676,7 +4143,7 @@
         <v/>
       </c>
       <c r="K13" s="11">
-        <f>IF($D13&lt;&gt;"yes","",Inputs!$B$60)</f>
+        <f>IF($D13&lt;&gt;"yes","",Inputs!$B$63)</f>
         <v/>
       </c>
       <c r="L13" s="11">
@@ -3684,7 +4151,7 @@
         <v/>
       </c>
       <c r="M13" s="11">
-        <f>IF($D13&lt;&gt;"yes","",Lines!$C$63)</f>
+        <f>IF($D13&lt;&gt;"yes","",Lines!$C$70)</f>
         <v/>
       </c>
       <c r="N13" s="11">
@@ -3715,11 +4182,11 @@
         <v/>
       </c>
       <c r="E14" s="11">
-        <f>IF($D14&lt;&gt;"yes","",Inputs!$B$4&amp;" – Last chance to "&amp;IF(Inputs!$B$12="draw","enter the draw","collect"))</f>
+        <f>IF($D14&lt;&gt;"yes","",Inputs!$B$4&amp;" – Last chance to "&amp;IF(Inputs!$B$14="draw","enter the draw","collect"))</f>
         <v/>
       </c>
       <c r="F14" s="11">
-        <f>IF($D14&lt;&gt;"yes","",IF(Inputs!$B$12="draw","The draw closes at "&amp;Inputs!$B$53&amp;" on "&amp;Inputs!$B$52&amp;".","Time is almost up."))</f>
+        <f>IF($D14&lt;&gt;"yes","",IF(Inputs!$B$14="draw","The draw closes at "&amp;Inputs!$B$56&amp;" on "&amp;Inputs!$B$55&amp;".","Time is almost up."))</f>
         <v/>
       </c>
       <c r="G14" s="11">
@@ -3727,19 +4194,19 @@
         <v/>
       </c>
       <c r="H14" s="11">
-        <f>IF($D14&lt;&gt;"yes","",IF(Inputs!$B$12="draw","Last chance to enter the draw","Last chance to collect"))</f>
+        <f>IF($D14&lt;&gt;"yes","",IF(Inputs!$B$14="draw","Last chance to enter the draw","Last chance to collect"))</f>
         <v/>
       </c>
       <c r="I14" s="11">
-        <f>IF($D14&lt;&gt;"yes","",IF(Inputs!$B$12="draw",(Lines!$C$67&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$68),(Lines!$C$65&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$66)))</f>
+        <f>IF($D14&lt;&gt;"yes","",IF(Inputs!$B$14="draw",(Lines!$C$74&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$30&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$75),(Lines!$C$72&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$73)))</f>
         <v/>
       </c>
       <c r="J14" s="11">
-        <f>IF($D14&lt;&gt;"yes","",IF(Inputs!$B$12="draw","Enter the draw","Buy now"))</f>
+        <f>IF($D14&lt;&gt;"yes","",IF(Inputs!$B$14="draw","Enter the draw","Buy now"))</f>
         <v/>
       </c>
       <c r="K14" s="11">
-        <f>IF($D14&lt;&gt;"yes","",Inputs!$B$60)</f>
+        <f>IF($D14&lt;&gt;"yes","",Inputs!$B$63)</f>
         <v/>
       </c>
       <c r="L14" s="11">
@@ -3774,11 +4241,11 @@
         </is>
       </c>
       <c r="D15" s="11">
-        <f>IF(Inputs!$B$12="draw","yes","(not used for a timed edition)")</f>
+        <f>IF(Inputs!$B$14="draw","yes","(not used for a timed edition)")</f>
         <v/>
       </c>
       <c r="E15" s="11">
-        <f>IF($D15&lt;&gt;"yes","",Lines!$C$70)</f>
+        <f>IF($D15&lt;&gt;"yes","",Lines!$C$77)</f>
         <v/>
       </c>
       <c r="F15" s="11">
@@ -3794,7 +4261,7 @@
         <v/>
       </c>
       <c r="I15" s="11">
-        <f>IF($D15&lt;&gt;"yes","",(Lines!$C$24&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$71&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$72&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$73&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$74))</f>
+        <f>IF($D15&lt;&gt;"yes","",(Lines!$C$31&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$78&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$79&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$80&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$81))</f>
         <v/>
       </c>
       <c r="J15" s="11">
@@ -3837,7 +4304,7 @@
         </is>
       </c>
       <c r="D16" s="11">
-        <f>IF(Inputs!$B$12="draw","yes","(not used for a timed edition)")</f>
+        <f>IF(Inputs!$B$14="draw","yes","(not used for a timed edition)")</f>
         <v/>
       </c>
       <c r="E16" s="11">
@@ -3857,7 +4324,7 @@
         <v/>
       </c>
       <c r="I16" s="11">
-        <f>IF($D16&lt;&gt;"yes","",(Lines!$C$75&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$76&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$77&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$78))</f>
+        <f>IF($D16&lt;&gt;"yes","",(Lines!$C$82&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$83&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$84&amp;CHAR(10)&amp;CHAR(10)&amp;Lines!$C$85))</f>
         <v/>
       </c>
       <c r="J16" s="11">
@@ -3873,7 +4340,7 @@
         <v/>
       </c>
       <c r="M16" s="11">
-        <f>IF($D16&lt;&gt;"yes","",Lines!$C$79)</f>
+        <f>IF($D16&lt;&gt;"yes","",Lines!$C$86)</f>
         <v/>
       </c>
       <c r="N16" s="11">
@@ -3920,7 +4387,7 @@
         <v/>
       </c>
       <c r="I17" s="11">
-        <f>IF($D17&lt;&gt;"yes","",(Lines!$C$81&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$28&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$46&amp;CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$12="draw",Lines!$C$82,Lines!$C$83)))</f>
+        <f>IF($D17&lt;&gt;"yes","",(Lines!$C$88&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$30&amp;CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$49&amp;CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$14="draw",Lines!$C$89,Lines!$C$90)))</f>
         <v/>
       </c>
       <c r="J17" s="11">
@@ -3953,13 +4420,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3981,7 +4448,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Every post on our own Instagram feed, and the emails in the comms plan: Announcement (TL and LE), Welcome, Early Access (TL Flow, TL Artist PP, Insiders TL and LE, LE early/exclusive), Now Live, Halfway, 5 days to go, 3 days to go, Last chance (TL and LE), the two LE surveys, and this release's paragraph for the Monthly Preview. The artist's own email is rare and stays hand-written.</t>
+          <t>Every post on our own Instagram feed and the Insiders account, the tweets, and the emails in the comms plan: Announcement (TL and LE), Welcome, Early Access (TL Flow, TL Artist PP, Insiders TL and LE, LE early/exclusive), Now Live, Halfway, 5 days to go, 3 days to go, Last chance (TL and LE), the two LE surveys, and this release's paragraph for the Monthly Preview. The artist's own email is rare and stays hand-written.</t>
         </is>
       </c>
     </row>
@@ -4000,118 +4467,142 @@
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>Skeleton, emails</t>
+          <t>Insiders</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Every email is: subject, preview, kicker, headline, body paragraphs, CTA, card, quote, footer. Bodies are fixed sentences from the Lines sheet with the same fragments dropped in. Halfway and 5 days to go have no body: they are image-led.</t>
+          <t>The Insiders account posts the same caption as the main feed. The plan says which: Announcement, Now Live and Halfway for a timed edition, Announcement for a draw. The Channels column on Posts carries this. Stories are image-led and stay outside the sheet.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>Fragments</t>
+          <t>Twitter</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Four per release, written once: bio (2 to 3 sentences, Coming Soon only), hook (1 to 2 sentences about the work, in every post and email), making (one sentence naming Make-Ready), quote (verbatim). The hook and bio must not repeat each other.</t>
+          <t>A tweet is the post's status line with the X handle, the hook on the announcement only, the beneficiary named once, and an action line that ends with the link: sign up for updates, enter the draw, or buy a print. No features line, no hashtag, no bio. Same deadline form. Coming soon names the artist and not the work.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Voice</t>
+          <t>Skeleton, emails</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Fragments are voice-neutral: no we or our, no artist name in the hook or the making line, and 'printmakers at Make-Ready'. The sheet adds 'our'. The Insiders email and the first-time survey are signed by the advisor named on Inputs. Features never say 'our'.</t>
+          <t>Every email is: subject, preview, kicker, headline, body paragraphs, CTA, card, quote, footer. Bodies are fixed sentences from the Lines sheet with the same fragments dropped in. Halfway and 5 days to go have no body: they are image-led.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Features</t>
+          <t>Fragments</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>The standard three (signed by the artist, individually numbered, free worldwide shipping) plus anything bespoke. One line of short sentences in a post, a list in an email. The beneficiary follows, named once.</t>
+          <t>Four per release, written once: bio (2 to 3 sentences, Coming Soon only), hook (1 to 2 sentences about the work, in every post and email), making (one sentence naming Make-Ready), quote (verbatim). The hook and bio must not repeat each other.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Beneficiary</t>
+          <t>Voice</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>One phrase everywhere: 'released in support of'. It goes in the opener unless the hook already names the beneficiary.</t>
+          <t>Fragments are voice-neutral: no we or our, no artist name in the hook or the making line, and 'printmakers at Make-Ready'. The sheet adds 'our'. The Insiders email and the first-time survey are signed by the advisor named on Inputs. Features never say 'our'.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="12" t="inlineStr">
         <is>
-          <t>Action lines</t>
+          <t>Features</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Three CTAs: get updates before launch, enter the draw for a draw, buy a print for an open window. One deadline form: Closes {date} at {time} UK time, or 'until {time} on {weekday}, {date}' in an email.</t>
+          <t>The standard three (signed by the artist, individually numbered, free worldwide shipping) plus anything bespoke. One line of short sentences in a post, a list in an email. The beneficiary follows, named once.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>Mechanic and window</t>
+          <t>Beneficiary</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Set mechanic to timed or draw and the sheet switches every line. For a timed edition, a 48-hour window gets the halfway email; a one-week window gets 5 days to go and 3 days to go.</t>
+          <t>One phrase everywhere: 'released in support of'. It goes in the opener unless the hook already names the beneficiary.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>Dates</t>
+          <t>Action lines</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Enter launch and close once as date and time; the sheet derives '30 April', '14:00 UK time', 'Thursday' and '07 May' where each email needs them.</t>
+          <t>Three CTAs: get updates before launch, enter the draw for a draw, buy a print for an open window. One deadline form: Closes {date} at {time} UK time, or 'until {time} on {weekday}, {date}' in an email.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>What stays written</t>
+          <t>Mechanic and window</t>
         </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>A delay reason, a framing paragraph, editorial deep dives, the rest of the Monthly Preview, the artist's own email, and anything for a second release.</t>
+          <t>Set mechanic to timed or draw and the sheet switches every line. For a timed edition, a 48-hour window gets the halfway email; a one-week window gets 5 days to go and 3 days to go.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
         <is>
+          <t>Dates</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Enter launch and close once as date and time; the sheet derives '30 April', '14:00 UK time', 'Thursday' and '07 May' where each email needs them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="46" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>What stays written</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>A delay reason, a framing paragraph, editorial deep dives, the rest of the Monthly Preview, the artist's own email, and anything for a second release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="46" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
           <t>How to use</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Fill the blue cells on Inputs. Read Posts and Emails. To change the house wording, edit the blue cells on Lines once.</t>
         </is>

</xml_diff>